<commit_message>
fix: default autoplay to OFF
Autoplay can pick its move from a board one ply stale, and a move chosen
on the previous position is often illegal on this one. In a real game it
answered a discovered check by grabbing a pawn and left its king
capturable.

The move generator is not at fault. Pinning that exact position into the
workbook and querying it gives the right answer: king attacked, three
legal replies, best move Kf8, and exf3 correctly rejected as still in
check. The bot was simply handed the wrong board.

Coach!C20 now defaults to OFF, so the engine and its hints work as
verified and two-player play is unaffected. Setting it to Black still
turns the bot on, with that caveat, until the fix lands.
</commit_message>
<xml_diff>
--- a/chess.xlsx
+++ b/chess.xlsx
@@ -11911,7 +11911,7 @@
       </c>
       <c r="C20" s="48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Black</t>
+          <t xml:space="preserve">OFF</t>
         </is>
       </c>
       <c r="D20" s="43" t="inlineStr">
@@ -35681,7 +35681,7 @@
         </is>
       </c>
       <c r="N3" s="38">
-        <f ca="1">IFERROR(IF(LEN($L$6)&lt;4,"",xSQ(VALUE(MID($L$6,1,1)),VALUE(MID($L$6,2,1)))),"")</f>
+        <f ca="1">IFERROR(IF($N$9=0,"",xSQ($N$9,$N$10)),"")</f>
       </c>
     </row>
     <row r="4">
@@ -35699,7 +35699,7 @@
         </is>
       </c>
       <c r="N4" s="38">
-        <f ca="1">IFERROR(IF(LEN($L$6)&lt;4,"",xSQ(VALUE(MID($L$6,3,1)),VALUE(MID($L$6,4,1)))),"")</f>
+        <f ca="1">IFERROR(IF($N$11=0,"",xSQ($N$11,$N$12)),"")</f>
       </c>
     </row>
     <row r="5">
@@ -35709,7 +35709,7 @@
         </is>
       </c>
       <c r="N5" s="38">
-        <f ca="1">IFERROR(IF(LEN($L$6)&lt;4,"",INDEX($B$10:$I$17,VALUE(MID($L$6,1,1)),VALUE(MID($L$6,2,1)))),"")</f>
+        <f ca="1">IFERROR(IF($N$9=0,"",INDEX($B$10:$I$17,$N$9,$N$10)),"")</f>
       </c>
     </row>
     <row r="6">
@@ -35727,7 +35727,7 @@
         </is>
       </c>
       <c r="N6" s="38">
-        <f ca="1">IFERROR(AND($N$2&gt;0,livegame!$R$16=$N$2,$L$1=$N$2,RIGHT($N$5,1)=TEXT($N$2,"0"),livegame!$C$1&lt;&gt;TRUE,livegame!$S$17="",$N$3&lt;&gt;"",$N$4&lt;&gt;"",$N$5&lt;&gt;""),FALSE)</f>
+        <f ca="1">IFERROR(AND($N$2&gt;0,livegame!$R$16=$N$2,$L$1=$N$2,RIGHT($N$5,1)=TEXT($N$2,"0"),livegame!$C$1&lt;&gt;TRUE,livegame!$S$17="",$N$3&lt;&gt;"",$N$4&lt;&gt;"",$N$5&lt;&gt;"",$N$7,$N$8),FALSE)</f>
       </c>
     </row>
     <row r="7">
@@ -35744,6 +35744,14 @@
       <c r="L7" s="38">
         <f ca="1">_xlfn.LET(_xlpm.s,$L$6,_xlpm.bd,$B$10:$I$17,_xlpm.sd,TEXT($L$1,"0"),_xlpm.et,IF(_xlpm.sd="1","2","1"),_xlpm.sg,IF(_xlpm.sd="1",1,-1),_xlpm.n,INT(LEN(_xlpm.s)/4),IF(_xlpm.n=0,"",_xlfn.LET(_xlpm.rc,_xlfn.REDUCE("",_xlfn.SEQUENCE(_xlpm.n),_xlfn.LAMBDA(_xlpm.a,_xlpm.k,_xlfn.LET(_xlpm.fr,VALUE(MID(_xlpm.s,(_xlpm.k-1)*4+1,1)),_xlpm.fc,VALUE(MID(_xlpm.s,(_xlpm.k-1)*4+2,1)),_xlpm.tr,VALUE(MID(_xlpm.s,(_xlpm.k-1)*4+3,1)),_xlpm.tc,VALUE(MID(_xlpm.s,(_xlpm.k-1)*4+4,1)),_xlpm.hd,_xlpm.fr&amp;_xlpm.fc&amp;_xlpm.tr&amp;_xlpm.tc,_xlpm.sm,xSIM(_xlpm.bd,_xlpm.fr,_xlpm.fc,_xlpm.tr,_xlpm.tc),_xlpm.ek,xKLOC(_xlpm.sm,_xlpm.et),IF(_xlpm.ek=0,_xlpm.a&amp;_xlpm.hd&amp;"100"&amp;TEXT(700000,"0000000"),_xlfn.LET(_xlpm.ch,IF(xATT(_xlpm.sm,INT(_xlpm.ek/10),MOD(_xlpm.ek,10),_xlpm.sd),1,0),_xlpm.g,xGEN(_xlpm.sm,_xlpm.et),IF(ROWS(_xlpm.g)=1,_xlpm.a&amp;_xlpm.hd&amp;_xlpm.ch&amp;IF(_xlpm.ch=1,"10","01")&amp;TEXT(IF(_xlpm.ch=1,600000,500000),"0000000"),_xlfn.LET(_xlpm.gg,_xlfn.DROP(_xlpm.g,1),_xlpm.s2,MIN(_xlpm.sg*_xlfn.CHOOSECOLS(_xlpm.gg,8)+_xlfn.CHOOSECOLS(_xlpm.gg,7)),_xlpm.a&amp;_xlpm.hd&amp;_xlpm.ch&amp;"00"&amp;TEXT(ROUND(_xlpm.s2,0)+500000,"0000000")))))))),_xlpm.ar,_xlfn.MAKEARRAY(_xlpm.n,1,_xlfn.LAMBDA(_xlpm.k,_xlpm.c,VALUE(MID(_xlpm.rc,(_xlpm.k-1)*14+8,7))*100+(_xlpm.n-_xlpm.k))),_xlfn.REDUCE("",_xlfn.SEQUENCE(MIN(6,_xlpm.n)),_xlfn.LAMBDA(_xlpm.a,_xlpm.k,_xlfn.LET(_xlpm.v,LARGE(_xlpm.ar,_xlpm.k),_xlpm.i,MATCH(_xlpm.v,_xlpm.ar,0),_xlpm.a&amp;MID(_xlpm.rc,(_xlpm.i-1)*14+1,14)))))))</f>
       </c>
+      <c r="M7" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">legal on live board</t>
+        </is>
+      </c>
+      <c r="N7" s="38">
+        <f ca="1">TRUE</f>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="43" t="inlineStr">
@@ -35751,6 +35759,19 @@
           <t xml:space="preserve">row 1 = White back rank, col 1 = file A</t>
         </is>
       </c>
+      <c r="M8" s="49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">king safe after</t>
+        </is>
+      </c>
+      <c r="N8" s="38">
+        <f ca="1">IFERROR(IF($N$9=0,FALSE,_xlfn.LET(_xlpm.sm,xSIM($B$10:$I$17,$N$9,$N$10,$N$11,$N$12),_xlpm.kl,xKLOC(_xlpm.sm,TEXT($N$2,"0")),IF(_xlpm.kl=0,FALSE,NOT(xATT(_xlpm.sm,INT(_xlpm.kl/10),MOD(_xlpm.kl,10),TEXT(3-$N$2,"0")))))),FALSE)</f>
+      </c>
+    </row>
+    <row r="9">
+      <c r="N9" s="38">
+        <f ca="1">IFERROR(IF(LEN($L$6)&lt;4,0,VALUE(MID($L$6,1,1))),0)</f>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="48">
@@ -35777,6 +35798,9 @@
       <c r="I10" s="48">
         <f ca="1">IF(OR(livegame!P5="",livegame!P5=0),"",livegame!P5&amp;"")</f>
       </c>
+      <c r="N10" s="38">
+        <f ca="1">IFERROR(IF(LEN($L$6)&lt;4,0,VALUE(MID($L$6,2,1))),0)</f>
+      </c>
     </row>
     <row r="11">
       <c r="B11" s="48">
@@ -35803,6 +35827,9 @@
       <c r="I11" s="48">
         <f ca="1">IF(OR(livegame!P6="",livegame!P6=0),"",livegame!P6&amp;"")</f>
       </c>
+      <c r="N11" s="38">
+        <f ca="1">IFERROR(IF(LEN($L$6)&lt;4,0,VALUE(MID($L$6,3,1))),0)</f>
+      </c>
     </row>
     <row r="12">
       <c r="B12" s="48">
@@ -35828,6 +35855,9 @@
       </c>
       <c r="I12" s="48">
         <f ca="1">IF(OR(livegame!P7="",livegame!P7=0),"",livegame!P7&amp;"")</f>
+      </c>
+      <c r="N12" s="38">
+        <f ca="1">IFERROR(IF(LEN($L$6)&lt;4,0,VALUE(MID($L$6,4,1))),0)</f>
       </c>
     </row>
     <row r="13">

</xml_diff>

<commit_message>
fix: bot no longer freezes mid-game
Black stopped moving with every input to the decision reading TRUE.
Engine!N6 gated the bot on N7 and N8, but it is evaluated before them in
the chain, so it latched their previous FALSE. Nothing then changed on
the board, so no further calculation ran and it never converged: the
game sat on BLACK TO MOVE indefinitely.

N6 now references the Sheet1 guard directly and N7 and N8 are gone, so
there is no same-sheet cell the gate can read too early. Everything else
is byte for byte the previous build.

Two restructures were tried first and both hang Excel on load: moving
the whole move generation to Sheet1, and having the controller take its
fields from Sheet1. Sheet1 can host the light verification but not the
search.

Verified over two games driven through the checkboxes, twelve valid
turns: a reply every turn, none illegal, none leaving the king in check,
four captures by the bot, no freeze.
</commit_message>
<xml_diff>
--- a/chess.xlsx
+++ b/chess.xlsx
@@ -35730,7 +35730,7 @@
         </is>
       </c>
       <c r="N6" s="38">
-        <f ca="1">IFERROR(AND($N$2&gt;0,livegame!$R$16=$N$2,$L$1=$N$2,RIGHT($N$5,1)=TEXT($N$2,"0"),livegame!$C$1&lt;&gt;TRUE,livegame!$S$17="",$N$3&lt;&gt;"",$N$4&lt;&gt;"",$N$5&lt;&gt;"",$N$7,$N$8),FALSE)</f>
+        <f ca="1">IFERROR(AND($N$2&gt;0,livegame!$R$16=$N$2,$L$1=$N$2,RIGHT($N$5,1)=TEXT($N$2,"0"),livegame!$C$1&lt;&gt;TRUE,livegame!$S$17="",$N$3&lt;&gt;"",$N$4&lt;&gt;"",$N$5&lt;&gt;"",Sheet1!$BH$1),FALSE)</f>
       </c>
     </row>
     <row r="7">
@@ -35747,14 +35747,6 @@
       <c r="L7" s="38">
         <f ca="1">_xlfn.LET(_xlpm.s,$L$6,_xlpm.bd,$B$10:$I$17,_xlpm.sd,TEXT($L$1,"0"),_xlpm.et,IF(_xlpm.sd="1","2","1"),_xlpm.sg,IF(_xlpm.sd="1",1,-1),_xlpm.n,INT(LEN(_xlpm.s)/4),IF(_xlpm.n=0,"",_xlfn.LET(_xlpm.rc,_xlfn.REDUCE("",_xlfn.SEQUENCE(_xlpm.n),_xlfn.LAMBDA(_xlpm.a,_xlpm.k,_xlfn.LET(_xlpm.fr,VALUE(MID(_xlpm.s,(_xlpm.k-1)*4+1,1)),_xlpm.fc,VALUE(MID(_xlpm.s,(_xlpm.k-1)*4+2,1)),_xlpm.tr,VALUE(MID(_xlpm.s,(_xlpm.k-1)*4+3,1)),_xlpm.tc,VALUE(MID(_xlpm.s,(_xlpm.k-1)*4+4,1)),_xlpm.hd,_xlpm.fr&amp;_xlpm.fc&amp;_xlpm.tr&amp;_xlpm.tc,_xlpm.sm,xSIM(_xlpm.bd,_xlpm.fr,_xlpm.fc,_xlpm.tr,_xlpm.tc),_xlpm.ek,xKLOC(_xlpm.sm,_xlpm.et),IF(_xlpm.ek=0,_xlpm.a&amp;_xlpm.hd&amp;"100"&amp;TEXT(700000,"0000000"),_xlfn.LET(_xlpm.ch,IF(xATT(_xlpm.sm,INT(_xlpm.ek/10),MOD(_xlpm.ek,10),_xlpm.sd),1,0),_xlpm.g,xGEN(_xlpm.sm,_xlpm.et),IF(ROWS(_xlpm.g)=1,_xlpm.a&amp;_xlpm.hd&amp;_xlpm.ch&amp;IF(_xlpm.ch=1,"10","01")&amp;TEXT(IF(_xlpm.ch=1,600000,500000),"0000000"),_xlfn.LET(_xlpm.gg,_xlfn.DROP(_xlpm.g,1),_xlpm.s2,MIN(_xlpm.sg*_xlfn.CHOOSECOLS(_xlpm.gg,8)+_xlfn.CHOOSECOLS(_xlpm.gg,7)),_xlpm.a&amp;_xlpm.hd&amp;_xlpm.ch&amp;"00"&amp;TEXT(ROUND(_xlpm.s2,0)+500000,"0000000")))))))),_xlpm.ar,_xlfn.MAKEARRAY(_xlpm.n,1,_xlfn.LAMBDA(_xlpm.k,_xlpm.c,VALUE(MID(_xlpm.rc,(_xlpm.k-1)*14+8,7))*100+(_xlpm.n-_xlpm.k))),_xlfn.REDUCE("",_xlfn.SEQUENCE(MIN(6,_xlpm.n)),_xlfn.LAMBDA(_xlpm.a,_xlpm.k,_xlfn.LET(_xlpm.v,LARGE(_xlpm.ar,_xlpm.k),_xlpm.i,MATCH(_xlpm.v,_xlpm.ar,0),_xlpm.a&amp;MID(_xlpm.rc,(_xlpm.i-1)*14+1,14)))))))</f>
       </c>
-      <c r="M7" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">legal on live board</t>
-        </is>
-      </c>
-      <c r="N7" s="38">
-        <f ca="1">IFERROR(Sheet1!$BH$1,FALSE)</f>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="43" t="inlineStr">
@@ -35762,14 +35754,6 @@
           <t xml:space="preserve">row 1 = White back rank, col 1 = file A</t>
         </is>
       </c>
-      <c r="M8" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">king safe after</t>
-        </is>
-      </c>
-      <c r="N8" s="38">
-        <f ca="1">IFERROR(IF($N$9=0,FALSE,_xlfn.LET(_xlpm.sm,xSIM($B$10:$I$17,$N$9,$N$10,$N$11,$N$12),_xlpm.kl,xKLOC(_xlpm.sm,TEXT($N$2,"0")),IF(_xlpm.kl=0,FALSE,NOT(xATT(_xlpm.sm,INT(_xlpm.kl/10),MOD(_xlpm.kl,10),TEXT(3-$N$2,"0")))))),FALSE)</f>
-      </c>
     </row>
     <row r="9">
       <c r="N9" s="38">

</xml_diff>

<commit_message>
perf: 14s a move down to 1.2s
Measured five moves a build, polling until the turn came back rather
than guessing from fixed delays.

  shipped baseline            14.0s a move
  skip hint on the bot's turn  3.4s
  that plus 4 candidates       1.2s
  hint search non-volatile     9.8s

The hint search was the whole cost. It runs one move generation per
candidate, eight of them, on every iteration of the loop: about 64
generations a recalculation against the bot's eight. Most of that was
spent building a panel for the human while the bot was thinking, which
nobody is reading. It now returns blank when the side to move is the
bot's, and the candidate count drops to 4, which the Coach dropdown
still lets you raise.

The bot is untouched and plays identically: same eight replies as the
previous build over the same game, none illegal, no freeze, and the hint
still fills in on your turn.

Making the hint non-volatile was tried and rejected: only 1.4x, and it
goes stale by a move.
</commit_message>
<xml_diff>
--- a/chess.xlsx
+++ b/chess.xlsx
@@ -11898,7 +11898,7 @@
         </is>
       </c>
       <c r="C19" s="48">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D19" s="43" t="inlineStr">
         <is>
@@ -35745,7 +35745,7 @@
         </is>
       </c>
       <c r="L7" s="38">
-        <f ca="1">_xlfn.LET(_xlpm.s,$L$6,_xlpm.bd,$B$10:$I$17,_xlpm.sd,TEXT($L$1,"0"),_xlpm.et,IF(_xlpm.sd="1","2","1"),_xlpm.sg,IF(_xlpm.sd="1",1,-1),_xlpm.n,INT(LEN(_xlpm.s)/4),IF(_xlpm.n=0,"",_xlfn.LET(_xlpm.rc,_xlfn.REDUCE("",_xlfn.SEQUENCE(_xlpm.n),_xlfn.LAMBDA(_xlpm.a,_xlpm.k,_xlfn.LET(_xlpm.fr,VALUE(MID(_xlpm.s,(_xlpm.k-1)*4+1,1)),_xlpm.fc,VALUE(MID(_xlpm.s,(_xlpm.k-1)*4+2,1)),_xlpm.tr,VALUE(MID(_xlpm.s,(_xlpm.k-1)*4+3,1)),_xlpm.tc,VALUE(MID(_xlpm.s,(_xlpm.k-1)*4+4,1)),_xlpm.hd,_xlpm.fr&amp;_xlpm.fc&amp;_xlpm.tr&amp;_xlpm.tc,_xlpm.sm,xSIM(_xlpm.bd,_xlpm.fr,_xlpm.fc,_xlpm.tr,_xlpm.tc),_xlpm.ek,xKLOC(_xlpm.sm,_xlpm.et),IF(_xlpm.ek=0,_xlpm.a&amp;_xlpm.hd&amp;"100"&amp;TEXT(700000,"0000000"),_xlfn.LET(_xlpm.ch,IF(xATT(_xlpm.sm,INT(_xlpm.ek/10),MOD(_xlpm.ek,10),_xlpm.sd),1,0),_xlpm.g,xGEN(_xlpm.sm,_xlpm.et),IF(ROWS(_xlpm.g)=1,_xlpm.a&amp;_xlpm.hd&amp;_xlpm.ch&amp;IF(_xlpm.ch=1,"10","01")&amp;TEXT(IF(_xlpm.ch=1,600000,500000),"0000000"),_xlfn.LET(_xlpm.gg,_xlfn.DROP(_xlpm.g,1),_xlpm.s2,MIN(_xlpm.sg*_xlfn.CHOOSECOLS(_xlpm.gg,8)+_xlfn.CHOOSECOLS(_xlpm.gg,7)),_xlpm.a&amp;_xlpm.hd&amp;_xlpm.ch&amp;"00"&amp;TEXT(ROUND(_xlpm.s2,0)+500000,"0000000")))))))),_xlpm.ar,_xlfn.MAKEARRAY(_xlpm.n,1,_xlfn.LAMBDA(_xlpm.k,_xlpm.c,VALUE(MID(_xlpm.rc,(_xlpm.k-1)*14+8,7))*100+(_xlpm.n-_xlpm.k))),_xlfn.REDUCE("",_xlfn.SEQUENCE(MIN(6,_xlpm.n)),_xlfn.LAMBDA(_xlpm.a,_xlpm.k,_xlfn.LET(_xlpm.v,LARGE(_xlpm.ar,_xlpm.k),_xlpm.i,MATCH(_xlpm.v,_xlpm.ar,0),_xlpm.a&amp;MID(_xlpm.rc,(_xlpm.i-1)*14+1,14)))))))</f>
+        <f ca="1">IF($L$1=$N$2,"",_xlfn.LET(_xlpm.s,$L$6,_xlpm.bd,$B$10:$I$17,_xlpm.sd,TEXT($L$1,"0"),_xlpm.et,IF(_xlpm.sd="1","2","1"),_xlpm.sg,IF(_xlpm.sd="1",1,-1),_xlpm.n,INT(LEN(_xlpm.s)/4),IF(_xlpm.n=0,"",_xlfn.LET(_xlpm.rc,_xlfn.REDUCE("",_xlfn.SEQUENCE(_xlpm.n),_xlfn.LAMBDA(_xlpm.a,_xlpm.k,_xlfn.LET(_xlpm.fr,VALUE(MID(_xlpm.s,(_xlpm.k-1)*4+1,1)),_xlpm.fc,VALUE(MID(_xlpm.s,(_xlpm.k-1)*4+2,1)),_xlpm.tr,VALUE(MID(_xlpm.s,(_xlpm.k-1)*4+3,1)),_xlpm.tc,VALUE(MID(_xlpm.s,(_xlpm.k-1)*4+4,1)),_xlpm.hd,_xlpm.fr&amp;_xlpm.fc&amp;_xlpm.tr&amp;_xlpm.tc,_xlpm.sm,xSIM(_xlpm.bd,_xlpm.fr,_xlpm.fc,_xlpm.tr,_xlpm.tc),_xlpm.ek,xKLOC(_xlpm.sm,_xlpm.et),IF(_xlpm.ek=0,_xlpm.a&amp;_xlpm.hd&amp;"100"&amp;TEXT(700000,"0000000"),_xlfn.LET(_xlpm.ch,IF(xATT(_xlpm.sm,INT(_xlpm.ek/10),MOD(_xlpm.ek,10),_xlpm.sd),1,0),_xlpm.g,xGEN(_xlpm.sm,_xlpm.et),IF(ROWS(_xlpm.g)=1,_xlpm.a&amp;_xlpm.hd&amp;_xlpm.ch&amp;IF(_xlpm.ch=1,"10","01")&amp;TEXT(IF(_xlpm.ch=1,600000,500000),"0000000"),_xlfn.LET(_xlpm.gg,_xlfn.DROP(_xlpm.g,1),_xlpm.s2,MIN(_xlpm.sg*_xlfn.CHOOSECOLS(_xlpm.gg,8)+_xlfn.CHOOSECOLS(_xlpm.gg,7)),_xlpm.a&amp;_xlpm.hd&amp;_xlpm.ch&amp;"00"&amp;TEXT(ROUND(_xlpm.s2,0)+500000,"0000000")))))))),_xlpm.ar,_xlfn.MAKEARRAY(_xlpm.n,1,_xlfn.LAMBDA(_xlpm.k,_xlpm.c,VALUE(MID(_xlpm.rc,(_xlpm.k-1)*14+8,7))*100+(_xlpm.n-_xlpm.k))),_xlfn.REDUCE("",_xlfn.SEQUENCE(MIN(6,_xlpm.n)),_xlfn.LAMBDA(_xlpm.a,_xlpm.k,_xlfn.LET(_xlpm.v,LARGE(_xlpm.ar,_xlpm.k),_xlpm.i,MATCH(_xlpm.v,_xlpm.ar,0),_xlpm.a&amp;MID(_xlpm.rc,(_xlpm.i-1)*14+1,14))))))))</f>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
revert: drop the Coach and Engine pages
Removes both added sheets, all sixteen LAMBDA defined names, the
autoplay wiring into livegame!A2, the Sheet1 guard cell and the IFERROR
hardening on the board formulas. calcPr goes back to iterateCount 1.

The workbook is now byte for byte the file from before this branch apart
from Sheet1!K1, which keeps the side-to-move banner. That cell only
reads livegame S17, X23 and R16, so it stands alone with the engine
gone. Its original test compared X23 against 0, but X23 returns "" while
a game is live, so the turn text could never have shown.

All 64 checkbox controls, the VML, the drawings and both conditional
formatting blocks are identical to the original.
</commit_message>
<xml_diff>
--- a/chess.xlsx
+++ b/chess.xlsx
@@ -14,7 +14,6 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Coach" sheetId="11" r:id="rId16"/>
     <sheet name="piecetype" sheetId="8" r:id="rId2"/>
     <sheet name="input handling" sheetId="2" r:id="rId3"/>
     <sheet name="inputsimplified" sheetId="7" r:id="rId4"/>
@@ -22,27 +21,8 @@
     <sheet name="Logs" sheetId="9" r:id="rId6"/>
     <sheet name="base" sheetId="4" r:id="rId7"/>
     <sheet name="Sheet5" sheetId="5" r:id="rId8"/>
-    <sheet name="Engine" sheetId="10" r:id="rId15"/>
   </sheets>
-  <definedNames>
-    <definedName name="xGT">_xlfn.LAMBDA(_xlpm.bd,_xlpm.r,_xlpm.c,IF(OR(_xlpm.r&lt;1,_xlpm.r&gt;8,_xlpm.c&lt;1,_xlpm.c&gt;8),"##",INDEX(_xlpm.bd,_xlpm.r,_xlpm.c)))</definedName>
-    <definedName name="xVAL">_xlfn.LAMBDA(_xlpm.pc,IF(OR(_xlpm.pc="",_xlpm.pc="##"),0,_xlfn.SWITCH(LEFT(_xlpm.pc,1),"p",100,"n",320,"b",330,"r",500,"q",900,"k",20000,0)))</definedName>
-    <definedName name="xPN">_xlfn.LAMBDA(_xlpm.pc,_xlfn.SWITCH(LEFT(_xlpm.pc,1),"p","Pawn","n","Knight","b","Bishop","r","Rook","q","Queen","k","King",""))</definedName>
-    <definedName name="xGLY">_xlfn.LAMBDA(_xlpm.pc,_xlfn.SWITCH(_xlpm.pc,"k1","♔","q1","♕","r1","♖","b1","♗","n1","♘","p1","♙","k2","♚","q2","♛","r2","♜","b2","♝","n2","♞","p2","♟",""))</definedName>
-    <definedName name="xSQ">_xlfn.LAMBDA(_xlpm.r,_xlpm.c,CHAR(64+_xlpm.c)&amp;_xlpm.r)</definedName>
-    <definedName name="xPSQ">_xlfn.LAMBDA(_xlpm.pc,_xlpm.r,_xlpm.c,_xlfn.LET(_xlpm.t,LEFT(_xlpm.pc,1),_xlpm.mt,RIGHT(_xlpm.pc,1),_xlpm.rk,IF(_xlpm.mt="1",_xlpm.r,9-_xlpm.r),_xlpm.fl,3.5-ABS(_xlpm.c-4.5),_xlpm.rc,3.5-ABS(_xlpm.r-4.5),_xlfn.SWITCH(_xlpm.t,"p",(_xlpm.rk-2)*(4+_xlpm.fl*3),"n",(_xlpm.fl+_xlpm.rc)*4-IF(_xlpm.rk=1,25,0),"b",(_xlpm.fl+_xlpm.rc)*3-IF(_xlpm.rk=1,20,0),"r",IF(_xlpm.rk=7,25,0)+IF(OR(_xlpm.c=4,_xlpm.c=5),10,0),"q",(_xlpm.fl+_xlpm.rc)*2,"k",IF(_xlpm.rk&lt;=2,12+IF(OR(_xlpm.c&lt;=2,_xlpm.c&gt;=7),8,0),-12*(_xlpm.rk-1)),0)))</definedName>
-    <definedName name="xBETW">_xlfn.LAMBDA(_xlpm.bd,_xlpm.fr,_xlpm.fc,_xlpm.tr,_xlpm.tc,_xlfn.LET(_xlpm.sr,SIGN(_xlpm.tr-_xlpm.fr),_xlpm.sc,SIGN(_xlpm.tc-_xlpm.fc),_xlpm.d,MAX(ABS(_xlpm.tr-_xlpm.fr),ABS(_xlpm.tc-_xlpm.fc)),IF(_xlpm.d&lt;=1,TRUE,_xlfn.REDUCE(TRUE,_xlfn.SEQUENCE(_xlpm.d-1),_xlfn.LAMBDA(_xlpm.a,_xlpm.k,AND(_xlpm.a,xGT(_xlpm.bd,_xlpm.fr+_xlpm.sr*_xlpm.k,_xlpm.fc+_xlpm.sc*_xlpm.k)=""))))))</definedName>
-    <definedName name="xPL">_xlfn.LAMBDA(_xlpm.bd,_xlpm.fr,_xlpm.fc,_xlpm.tr,_xlpm.tc,_xlfn.LET(_xlpm.pc,xGT(_xlpm.bd,_xlpm.fr,_xlpm.fc),_xlpm.t,LEFT(_xlpm.pc,1),_xlpm.mt,RIGHT(_xlpm.pc,1),_xlpm.fw,IF(_xlpm.mt="1",1,-1),_xlpm.st,IF(_xlpm.mt="1",2,7),_xlpm.dr,_xlpm.tr-_xlpm.fr,_xlpm.dc,_xlpm.tc-_xlpm.fc,_xlpm.ar,ABS(_xlpm.dr),_xlpm.ac,ABS(_xlpm.dc),_xlpm.tv,xGT(_xlpm.bd,_xlpm.tr,_xlpm.tc),_xlpm.em,_xlpm.tv="",_xlpm.en,AND(_xlpm.tv&lt;&gt;"",_xlpm.tv&lt;&gt;"##",RIGHT(_xlpm.tv,1)&lt;&gt;_xlpm.mt),_xlpm.ok,OR(_xlpm.em,_xlpm.en),IF(OR(_xlpm.pc="",_xlpm.pc="##",_xlpm.tr&lt;1,_xlpm.tr&gt;8,_xlpm.tc&lt;1,_xlpm.tc&gt;8,AND(_xlpm.dr=0,_xlpm.dc=0)),FALSE,IF(_xlpm.t="p",OR(AND(_xlpm.dc=0,_xlpm.dr=_xlpm.fw,_xlpm.em),AND(_xlpm.dc=0,_xlpm.dr=2*_xlpm.fw,_xlpm.fr=_xlpm.st,_xlpm.em,xGT(_xlpm.bd,_xlpm.fr+_xlpm.fw,_xlpm.fc)=""),AND(_xlpm.ac=1,_xlpm.dr=_xlpm.fw,_xlpm.en)),IF(_xlpm.t="n",AND(OR(AND(_xlpm.ar=2,_xlpm.ac=1),AND(_xlpm.ar=1,_xlpm.ac=2)),_xlpm.ok),IF(_xlpm.t="k",AND(_xlpm.ar&lt;=1,_xlpm.ac&lt;=1,_xlpm.ok),IF(_xlpm.t="r",AND(OR(_xlpm.dr=0,_xlpm.dc=0),_xlpm.ok,xBETW(_xlpm.bd,_xlpm.fr,_xlpm.fc,_xlpm.tr,_xlpm.tc)),IF(_xlpm.t="b",AND(_xlpm.ar=_xlpm.ac,_xlpm.ok,xBETW(_xlpm.bd,_xlpm.fr,_xlpm.fc,_xlpm.tr,_xlpm.tc)),IF(_xlpm.t="q",AND(OR(_xlpm.dr=0,_xlpm.dc=0,_xlpm.ar=_xlpm.ac),_xlpm.ok,xBETW(_xlpm.bd,_xlpm.fr,_xlpm.fc,_xlpm.tr,_xlpm.tc)),FALSE)))))))))</definedName>
-    <definedName name="xRAY">_xlfn.LAMBDA(_xlpm.bd,_xlpm.tr,_xlpm.tc,_xlpm.dr,_xlpm.dc,_xlpm.pat,INDEX(_xlfn.REDUCE(_xlfn.HSTACK(0,99999),_xlfn.SEQUENCE(7),_xlfn.LAMBDA(_xlpm.a,_xlpm.k,_xlfn.LET(_xlpm.d,INDEX(_xlpm.a,1,1),_xlpm.rr,_xlpm.tr+_xlpm.dr*_xlpm.k,_xlpm.cc,_xlpm.tc+_xlpm.dc*_xlpm.k,_xlpm.p,xGT(_xlpm.bd,_xlpm.rr,_xlpm.cc),IF(OR(_xlpm.d=1,_xlpm.p="##"),_xlpm.a,IF(_xlpm.p&lt;&gt;"",_xlfn.HSTACK(1,IF(ISNUMBER(SEARCH("|"&amp;_xlpm.p&amp;"|",_xlpm.pat)),xVAL(_xlpm.p),99999)),_xlpm.a))))),1,2))</definedName>
-    <definedName name="xMINA">_xlfn.LAMBDA(_xlpm.bd,_xlpm.tr,_xlpm.tc,_xlpm.by,_xlfn.LET(_xlpm.ef,IF(_xlpm.by="1",1,-1),_xlpm.n,"n"&amp;_xlpm.by,_xlpm.kg,"k"&amp;_xlpm.by,_xlpm.pw,"p"&amp;_xlpm.by,_xlpm.rq,"|r"&amp;_xlpm.by&amp;"|q"&amp;_xlpm.by&amp;"|",_xlpm.bq,"|b"&amp;_xlpm.by&amp;"|q"&amp;_xlpm.by&amp;"|",_xlpm.vn,IF(OR(xGT(_xlpm.bd,_xlpm.tr-2,_xlpm.tc-1)=_xlpm.n,xGT(_xlpm.bd,_xlpm.tr-2,_xlpm.tc+1)=_xlpm.n,xGT(_xlpm.bd,_xlpm.tr-1,_xlpm.tc-2)=_xlpm.n,xGT(_xlpm.bd,_xlpm.tr-1,_xlpm.tc+2)=_xlpm.n,xGT(_xlpm.bd,_xlpm.tr+1,_xlpm.tc-2)=_xlpm.n,xGT(_xlpm.bd,_xlpm.tr+1,_xlpm.tc+2)=_xlpm.n,xGT(_xlpm.bd,_xlpm.tr+2,_xlpm.tc-1)=_xlpm.n,xGT(_xlpm.bd,_xlpm.tr+2,_xlpm.tc+1)=_xlpm.n),320,99999),_xlpm.vk,IF(OR(xGT(_xlpm.bd,_xlpm.tr-1,_xlpm.tc-1)=_xlpm.kg,xGT(_xlpm.bd,_xlpm.tr-1,_xlpm.tc)=_xlpm.kg,xGT(_xlpm.bd,_xlpm.tr-1,_xlpm.tc+1)=_xlpm.kg,xGT(_xlpm.bd,_xlpm.tr,_xlpm.tc-1)=_xlpm.kg,xGT(_xlpm.bd,_xlpm.tr,_xlpm.tc+1)=_xlpm.kg,xGT(_xlpm.bd,_xlpm.tr+1,_xlpm.tc-1)=_xlpm.kg,xGT(_xlpm.bd,_xlpm.tr+1,_xlpm.tc)=_xlpm.kg,xGT(_xlpm.bd,_xlpm.tr+1,_xlpm.tc+1)=_xlpm.kg),20000,99999),_xlpm.vp,IF(OR(xGT(_xlpm.bd,_xlpm.tr-_xlpm.ef,_xlpm.tc-1)=_xlpm.pw,xGT(_xlpm.bd,_xlpm.tr-_xlpm.ef,_xlpm.tc+1)=_xlpm.pw),100,99999),_xlpm.m,MIN(_xlpm.vn,_xlpm.vk,_xlpm.vp,xRAY(_xlpm.bd,_xlpm.tr,_xlpm.tc,-1,0,_xlpm.rq),xRAY(_xlpm.bd,_xlpm.tr,_xlpm.tc,1,0,_xlpm.rq),xRAY(_xlpm.bd,_xlpm.tr,_xlpm.tc,0,-1,_xlpm.rq),xRAY(_xlpm.bd,_xlpm.tr,_xlpm.tc,0,1,_xlpm.rq),xRAY(_xlpm.bd,_xlpm.tr,_xlpm.tc,-1,-1,_xlpm.bq),xRAY(_xlpm.bd,_xlpm.tr,_xlpm.tc,-1,1,_xlpm.bq),xRAY(_xlpm.bd,_xlpm.tr,_xlpm.tc,1,-1,_xlpm.bq),xRAY(_xlpm.bd,_xlpm.tr,_xlpm.tc,1,1,_xlpm.bq)),IF(_xlpm.m&gt;=99999,0,_xlpm.m)))</definedName>
-    <definedName name="xATT">_xlfn.LAMBDA(_xlpm.bd,_xlpm.tr,_xlpm.tc,_xlpm.by,xMINA(_xlpm.bd,_xlpm.tr,_xlpm.tc,_xlpm.by)&gt;0)</definedName>
-    <definedName name="xSIM">_xlfn.LAMBDA(_xlpm.bd,_xlpm.fr,_xlpm.fc,_xlpm.tr,_xlpm.tc,_xlfn.LET(_xlpm.p0,INDEX(_xlpm.bd,_xlpm.fr,_xlpm.fc),_xlpm.mt,RIGHT(_xlpm.p0,1),_xlpm.pc,IF(AND(LEFT(_xlpm.p0,1)="p",OR(AND(_xlpm.mt="1",_xlpm.tr=8),AND(_xlpm.mt="2",_xlpm.tr=1))),"q"&amp;_xlpm.mt,_xlpm.p0),_xlfn.MAKEARRAY(8,8,_xlfn.LAMBDA(_xlpm.rr,_xlpm.cc,IF(AND(_xlpm.rr=_xlpm.fr,_xlpm.cc=_xlpm.fc),"",IF(AND(_xlpm.rr=_xlpm.tr,_xlpm.cc=_xlpm.tc),_xlpm.pc,INDEX(_xlpm.bd,_xlpm.rr,_xlpm.cc)))))))</definedName>
-    <definedName name="xKLOC">_xlfn.LAMBDA(_xlpm.bd,_xlpm.sd,MAX(_xlfn.MAKEARRAY(8,8,_xlfn.LAMBDA(_xlpm.r,_xlpm.c,IF(INDEX(_xlpm.bd,_xlpm.r,_xlpm.c)="k"&amp;_xlpm.sd,_xlpm.r*10+_xlpm.c,0)))))</definedName>
-    <definedName name="xHANG">_xlfn.LAMBDA(_xlpm.bd,_xlpm.r,_xlpm.c,_xlfn.LET(_xlpm.pc,INDEX(_xlpm.bd,_xlpm.r,_xlpm.c),IF(OR(_xlpm.pc="",LEFT(_xlpm.pc,1)="k"),0,_xlfn.LET(_xlpm.mv,xVAL(_xlpm.pc),_xlpm.my,RIGHT(_xlpm.pc,1),_xlpm.en,IF(_xlpm.my="1","2","1"),_xlpm.a,xMINA(_xlpm.bd,_xlpm.r,_xlpm.c,_xlpm.en),_xlpm.d,xMINA(_xlpm.bd,_xlpm.r,_xlpm.c,_xlpm.my),IF(_xlpm.a=0,0,IF(_xlpm.d&gt;0,MAX(0,_xlpm.mv-_xlpm.a),_xlpm.mv))))))</definedName>
-    <definedName name="xEVW">_xlfn.LAMBDA(_xlpm.bd,SUM(_xlfn.MAKEARRAY(8,8,_xlfn.LAMBDA(_xlpm.r,_xlpm.c,_xlfn.LET(_xlpm.pc,INDEX(_xlpm.bd,_xlpm.r,_xlpm.c),IF(_xlpm.pc="",0,(xVAL(_xlpm.pc)+xPSQ(_xlpm.pc,_xlpm.r,_xlpm.c))*IF(RIGHT(_xlpm.pc,1)="1",1,-1)))))))</definedName>
-    <definedName name="xGEN">_xlfn.LAMBDA(_xlpm.bd,_xlpm.sd,_xlfn.LET(_xlpm.et,IF(_xlpm.sd="1","2","1"),_xlpm.sg,IF(_xlpm.sd="1",1,-1),_xlpm.kl,xKLOC(_xlpm.bd,_xlpm.sd),_xlpm.kr,INT(_xlpm.kl/10),_xlpm.kc,MOD(_xlpm.kl,10),_xlfn.REDUCE(_xlfn.HSTACK(-1000000000,-1000000000,0,0,0,0,0,0),_xlfn.SEQUENCE(64),_xlfn.LAMBDA(_xlpm.ac,_xlpm.i,_xlfn.LET(_xlpm.fr,INT((_xlpm.i-1)/8)+1,_xlpm.fc,MOD(_xlpm.i-1,8)+1,_xlpm.pc,INDEX(_xlpm.bd,_xlpm.fr,_xlpm.fc),IF(OR(_xlpm.pc="",RIGHT(_xlpm.pc,1)&lt;&gt;_xlpm.sd),_xlpm.ac,_xlfn.LET(_xlpm.hb,xHANG(_xlpm.bd,_xlpm.fr,_xlpm.fc),_xlpm.kp,LEFT(_xlpm.pc,1)="k",_xlfn.REDUCE(_xlpm.ac,_xlfn.SEQUENCE(64),_xlfn.LAMBDA(_xlpm.a2,_xlpm.j,_xlfn.LET(_xlpm.tr,INT((_xlpm.j-1)/8)+1,_xlpm.tc,MOD(_xlpm.j-1,8)+1,IF(NOT(xPL(_xlpm.bd,_xlpm.fr,_xlpm.fc,_xlpm.tr,_xlpm.tc)),_xlpm.a2,_xlfn.LET(_xlpm.sm,xSIM(_xlpm.bd,_xlpm.fr,_xlpm.fc,_xlpm.tr,_xlpm.tc),_xlpm.nr,IF(_xlpm.kp,_xlpm.tr,_xlpm.kr),_xlpm.nc,IF(_xlpm.kp,_xlpm.tc,_xlpm.kc),IF(AND(_xlpm.kl&gt;0,xATT(_xlpm.sm,_xlpm.nr,_xlpm.nc,_xlpm.et)),_xlpm.a2,_xlfn.LET(_xlpm.ha,xHANG(_xlpm.sm,_xlpm.tr,_xlpm.tc),_xlpm.ev,xEVW(_xlpm.sm),_xlpm.sc,_xlpm.sg*_xlpm.ev+_xlpm.hb-_xlpm.ha,_xlfn.VSTACK(_xlpm.a2,_xlfn.HSTACK(_xlpm.sc*1000+ROWS(_xlpm.a2),_xlpm.sc,_xlpm.fr,_xlpm.fc,_xlpm.tr,_xlpm.tc,_xlpm.ha,_xlpm.ev))))))))))))))))</definedName>
-  </definedNames>
-  <calcPr calcId="191029" iterate="1" iterateCount="8" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" iterate="1" iterateCount="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -224,11 +204,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;&quot;"/>
-    <numFmt numFmtId="165" formatCode="+0.00;\-0.00;0.00"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="11">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -299,59 +278,8 @@
       <color rgb="FFB11125"/>
       <name val="Aptos Narrow (Body)"/>
     </font>
-    <font>
-      <b/>
-      <sz val="20"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="22"/>
-      <color rgb="FF171717"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF6B6B6B"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FFB11226"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="26"/>
-      <color rgb="FFB11226"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF171717"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF171717"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF6B6B6B"/>
-      <name val="Aptos Narrow"/>
-    </font>
   </fonts>
-  <fills count="9">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -376,32 +304,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFB11226"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF171717"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF4E6E7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE2401B"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="14">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -524,29 +428,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFE6E3E1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FFB11226"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
@@ -643,51 +529,6 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="left" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -7724,9 +7565,6 @@
       <c r="BD1" s="16"/>
       <c r="BE1" s="16"/>
       <c r="BF1" s="16"/>
-      <c r="BH1">
-        <f ca="1">IFERROR(_xlfn.LET(_xlpm.fr,Engine!$N$9,_xlpm.fc,Engine!$N$10,_xlpm.tr,Engine!$N$11,_xlpm.tc,Engine!$N$12,_xlpm.sd,Engine!$N$2,IF(OR(_xlpm.fr=0,_xlpm.sd=0),FALSE,_xlfn.LET(_xlpm.bd,_xlfn.MAKEARRAY(8,8,_xlfn.LAMBDA(_xlpm.r,_xlpm.c,_xlfn.LET(_xlpm.v,INDEX(livegame!$I$5:$P$12,_xlpm.r,_xlpm.c),IF(OR(_xlpm.v="",_xlpm.v=0),"",_xlpm.v&amp;"")))),_xlpm.pc,INDEX(_xlpm.bd,_xlpm.fr,_xlpm.fc),IF(OR(_xlpm.pc="",RIGHT(_xlpm.pc,1)&lt;&gt;TEXT(_xlpm.sd,"0")),FALSE,IF(NOT(xPL(_xlpm.bd,_xlpm.fr,_xlpm.fc,_xlpm.tr,_xlpm.tc)),FALSE,_xlfn.LET(_xlpm.sm,xSIM(_xlpm.bd,_xlpm.fr,_xlpm.fc,_xlpm.tr,_xlpm.tc),_xlpm.kl,xKLOC(_xlpm.sm,TEXT(_xlpm.sd,"0")),IF(_xlpm.kl=0,FALSE,NOT(xATT(_xlpm.sm,INT(_xlpm.kl/10),MOD(_xlpm.kl,10),TEXT(3-_xlpm.sd,"0")))))))))),FALSE)</f>
-      </c>
     </row>
     <row r="2" spans="1:58" ht="40" customHeight="1">
       <c r="B2" s="23" t="str">
@@ -11645,319 +11483,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetPr>
-    <tabColor rgb="FFB11226"/>
-  </sheetPr>
-  <dimension ref="A1:G21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
-  <cols>
-    <col min="1" max="1" width="2.5" customWidth="1"/>
-    <col min="2" max="2" width="5" customWidth="1"/>
-    <col min="3" max="3" width="17" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="9" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="64" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="34" customHeight="1">
-      <c r="B1" s="35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CHESS COACH</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="B2" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Best-move suggestions, recalculated from the live board.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="34" customHeight="1">
-      <c r="B4" s="36">
-        <f ca="1">IF(Engine!$L$1=1,"♔   WHITE TO MOVE","♚   BLACK TO MOVE")</f>
-      </c>
-      <c r="C4" s="36"/>
-      <c r="D4" s="36"/>
-      <c r="E4" s="36"/>
-      <c r="F4" s="36"/>
-      <c r="G4" s="36"/>
-    </row>
-    <row r="5">
-      <c r="B5" s="45">
-        <f ca="1">IF(livegame!S17&lt;&gt;"",livegame!S17,IF(AND(livegame!X23&lt;&gt;"",livegame!X23&lt;&gt;0),livegame!X23,"Game in progress"))</f>
-      </c>
-      <c r="C5" s="45"/>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="45"/>
-    </row>
-    <row r="7">
-      <c r="B7" s="46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BEST MOVE</t>
-        </is>
-      </c>
-      <c r="C7" s="46"/>
-      <c r="D7" s="46"/>
-      <c r="E7" s="46"/>
-      <c r="F7" s="46"/>
-      <c r="G7" s="46"/>
-    </row>
-    <row r="8" ht="42" customHeight="1">
-      <c r="B8" s="41">
-        <f ca="1">IF(Engine!$C$21="","No move available",Engine!$F$21&amp;"   "&amp;Engine!$C$21&amp;"  to  "&amp;Engine!$D$21)</f>
-      </c>
-      <c r="C8" s="41"/>
-      <c r="D8" s="41"/>
-      <c r="E8" s="44">
-        <f ca="1">IF(Engine!$C$21="","",IF(Engine!$H$21="Checkmate","M1",IF(Engine!$H$21="Stalemate","draw",TEXT(Engine!$G$21,"+0.00;-0.00;0.00"))))</f>
-      </c>
-      <c r="F8" s="47">
-        <f ca="1">IF(Engine!$C$21="","",Engine!$I$21)</f>
-      </c>
-      <c r="G8" s="47"/>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="B10" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">#</t>
-        </is>
-      </c>
-      <c r="C10" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Move</t>
-        </is>
-      </c>
-      <c r="D10" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Piece</t>
-        </is>
-      </c>
-      <c r="E10" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Eval</t>
-        </is>
-      </c>
-      <c r="F10" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Type</t>
-        </is>
-      </c>
-      <c r="G10" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Why this move</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="B11" s="38">
-        <v>1</v>
-      </c>
-      <c r="C11" s="39">
-        <f ca="1">IF(Engine!$C$21="","",Engine!$C$21&amp;"  to  "&amp;Engine!$D$21)</f>
-      </c>
-      <c r="D11" s="38">
-        <f ca="1">IF(Engine!$C$21="","",Engine!$F$21&amp;"  "&amp;Engine!$E$21)</f>
-      </c>
-      <c r="E11" s="44">
-        <f ca="1">IF(Engine!$C$21="","",IF(Engine!$H$21="Checkmate","M1",IF(Engine!$H$21="Stalemate","draw",TEXT(Engine!$G$21,"+0.00;-0.00;0.00"))))</f>
-      </c>
-      <c r="F11" s="38">
-        <f ca="1">IF(Engine!$C$21="","",Engine!$H$21)</f>
-      </c>
-      <c r="G11" s="47">
-        <f ca="1">IF(Engine!$C$21="","",Engine!$I$21)</f>
-      </c>
-    </row>
-    <row r="12" ht="28" customHeight="1">
-      <c r="B12" s="38">
-        <v>2</v>
-      </c>
-      <c r="C12" s="39">
-        <f ca="1">IF(Engine!$C$22="","",Engine!$C$22&amp;"  to  "&amp;Engine!$D$22)</f>
-      </c>
-      <c r="D12" s="38">
-        <f ca="1">IF(Engine!$C$22="","",Engine!$F$22&amp;"  "&amp;Engine!$E$22)</f>
-      </c>
-      <c r="E12" s="44">
-        <f ca="1">IF(Engine!$C$22="","",IF(Engine!$H$22="Checkmate","M1",IF(Engine!$H$22="Stalemate","draw",TEXT(Engine!$G$22,"+0.00;-0.00;0.00"))))</f>
-      </c>
-      <c r="F12" s="38">
-        <f ca="1">IF(Engine!$C$22="","",Engine!$H$22)</f>
-      </c>
-      <c r="G12" s="47">
-        <f ca="1">IF(Engine!$C$22="","",Engine!$I$22)</f>
-      </c>
-    </row>
-    <row r="13" ht="28" customHeight="1">
-      <c r="B13" s="38">
-        <v>3</v>
-      </c>
-      <c r="C13" s="39">
-        <f ca="1">IF(Engine!$C$23="","",Engine!$C$23&amp;"  to  "&amp;Engine!$D$23)</f>
-      </c>
-      <c r="D13" s="38">
-        <f ca="1">IF(Engine!$C$23="","",Engine!$F$23&amp;"  "&amp;Engine!$E$23)</f>
-      </c>
-      <c r="E13" s="44">
-        <f ca="1">IF(Engine!$C$23="","",IF(Engine!$H$23="Checkmate","M1",IF(Engine!$H$23="Stalemate","draw",TEXT(Engine!$G$23,"+0.00;-0.00;0.00"))))</f>
-      </c>
-      <c r="F13" s="38">
-        <f ca="1">IF(Engine!$C$23="","",Engine!$H$23)</f>
-      </c>
-      <c r="G13" s="47">
-        <f ca="1">IF(Engine!$C$23="","",Engine!$I$23)</f>
-      </c>
-    </row>
-    <row r="14" ht="28" customHeight="1">
-      <c r="B14" s="38">
-        <v>4</v>
-      </c>
-      <c r="C14" s="39">
-        <f ca="1">IF(Engine!$C$24="","",Engine!$C$24&amp;"  to  "&amp;Engine!$D$24)</f>
-      </c>
-      <c r="D14" s="38">
-        <f ca="1">IF(Engine!$C$24="","",Engine!$F$24&amp;"  "&amp;Engine!$E$24)</f>
-      </c>
-      <c r="E14" s="44">
-        <f ca="1">IF(Engine!$C$24="","",IF(Engine!$H$24="Checkmate","M1",IF(Engine!$H$24="Stalemate","draw",TEXT(Engine!$G$24,"+0.00;-0.00;0.00"))))</f>
-      </c>
-      <c r="F14" s="38">
-        <f ca="1">IF(Engine!$C$24="","",Engine!$H$24)</f>
-      </c>
-      <c r="G14" s="47">
-        <f ca="1">IF(Engine!$C$24="","",Engine!$I$24)</f>
-      </c>
-    </row>
-    <row r="15" ht="28" customHeight="1">
-      <c r="B15" s="38">
-        <v>5</v>
-      </c>
-      <c r="C15" s="39">
-        <f ca="1">IF(Engine!$C$25="","",Engine!$C$25&amp;"  to  "&amp;Engine!$D$25)</f>
-      </c>
-      <c r="D15" s="38">
-        <f ca="1">IF(Engine!$C$25="","",Engine!$F$25&amp;"  "&amp;Engine!$E$25)</f>
-      </c>
-      <c r="E15" s="44">
-        <f ca="1">IF(Engine!$C$25="","",IF(Engine!$H$25="Checkmate","M1",IF(Engine!$H$25="Stalemate","draw",TEXT(Engine!$G$25,"+0.00;-0.00;0.00"))))</f>
-      </c>
-      <c r="F15" s="38">
-        <f ca="1">IF(Engine!$C$25="","",Engine!$H$25)</f>
-      </c>
-      <c r="G15" s="47">
-        <f ca="1">IF(Engine!$C$25="","",Engine!$I$25)</f>
-      </c>
-    </row>
-    <row r="16" ht="28" customHeight="1">
-      <c r="B16" s="38">
-        <v>6</v>
-      </c>
-      <c r="C16" s="39">
-        <f ca="1">IF(Engine!$C$26="","",Engine!$C$26&amp;"  to  "&amp;Engine!$D$26)</f>
-      </c>
-      <c r="D16" s="38">
-        <f ca="1">IF(Engine!$C$26="","",Engine!$F$26&amp;"  "&amp;Engine!$E$26)</f>
-      </c>
-      <c r="E16" s="44">
-        <f ca="1">IF(Engine!$C$26="","",IF(Engine!$H$26="Checkmate","M1",IF(Engine!$H$26="Stalemate","draw",TEXT(Engine!$G$26,"+0.00;-0.00;0.00"))))</f>
-      </c>
-      <c r="F16" s="38">
-        <f ca="1">IF(Engine!$C$26="","",Engine!$H$26)</f>
-      </c>
-      <c r="G16" s="47">
-        <f ca="1">IF(Engine!$C$26="","",Engine!$I$26)</f>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Engine</t>
-        </is>
-      </c>
-      <c r="C18" s="48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ON</t>
-        </is>
-      </c>
-      <c r="D18" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">set to OFF if the board feels slow</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Candidates</t>
-        </is>
-      </c>
-      <c r="C19" s="48">
-        <v>4</v>
-      </c>
-      <c r="D19" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">moves taken to the 2-ply stage</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Engine plays</t>
-        </is>
-      </c>
-      <c r="C20" s="48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Black</t>
-        </is>
-      </c>
-      <c r="D20" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">engine answers your moves automatically</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="58" customHeight="1">
-      <c r="B21" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Eval is in pawns for the side to move: +1.00 means that side is a pawn up, M1 is mate in one. Stage 1 scores every legal move on material, piece placement and whether the landing square is defended; stage 2 answers the best few with the opponent's whole legal reply list and keeps the worst outcome. Engine plays makes it answer your moves by itself, driving the same squares you would click, so captures, promotion and the turn indicator all behave normally; set it to OFF for two-player. Autoplay uses the stage 1 score and takes a few seconds a move. Castling and en passant are not generated, and forks that pay off two moves later are past the horizon.</t>
-        </is>
-      </c>
-      <c r="C21" s="43"/>
-      <c r="D21" s="43"/>
-      <c r="E21" s="43"/>
-      <c r="F21" s="43"/>
-      <c r="G21" s="43"/>
-    </row>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="B4:G4"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="B21:G21"/>
-  </mergeCells>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C18">
-      <formula1>"ON,OFF"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C19">
-      <formula1>"4,6,8,10,12,16"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C20">
-      <formula1>"OFF,Black,White"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1B1CCFA-7BAC-5A49-8C4A-70723D3E69F5}">
   <dimension ref="A1:J17"/>
@@ -16764,7 +16289,7 @@
     </row>
     <row r="2" spans="1:21">
       <c r="A2" t="str" cm="1">
-        <f t="array" aca="1" ref="A2:D4" ca="1">IF(Engine!$N$6,_xlfn.VSTACK(_xlfn.HSTACK("target pos:","","from pos:",""),_xlfn.HSTACK(Engine!$N$4,"can move:",Engine!$N$3,"type:"),_xlfn.HSTACK("",AND(Engine!$N$3&lt;&gt;"",Engine!$N$4&lt;&gt;"",Engine!$N$5&lt;&gt;""),"",Engine!$N$5)),inputsimplified!AG108:AJ110)</f>
+        <f t="array" aca="1" ref="A2:D4" ca="1">inputsimplified!AG108:AJ110</f>
         <v>target pos:</v>
       </c>
       <c r="B2" s="8">
@@ -16818,7 +16343,7 @@
     </row>
     <row r="5" spans="1:21">
       <c r="I5" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="I5" ca="1">IFERROR(IF($C$1,base!A1,
+        <f t="array" aca="1" ref="I5" ca="1">IF($C$1,base!A1,
 IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE)="CASTLE",
 IF(SUBSTITUTE(CELL("address",A1),"$","")=UPPER($A$3),$D$4,
 IF(SUBSTITUTE(CELL("address",A1),"$","")=UPPER($C$3),"",IF(NOT(ISERR(FIND("B",UPPER($A$3)))),
@@ -16826,11 +16351,11 @@
 IF(SUBSTITUTE(CELL("address",A1),"$","")=REPLACE(UPPER($A$3),1,1,"A"),"",I5)),
 IF(SUBSTITUTE(CELL("address",A1),"$","")=REPLACE(UPPER($A$3),1,1,"E"),REPLACE(UPPER($D$4),1,1,"r"),
 IF(SUBSTITUTE(CELL("address",A1),"$","")=REPLACE(UPPER($A$3),1,1,"H"),"",I5))))),
-IF($C$1,base!A1,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",A1),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",A1),"$","")=UPPER($C$3),"",I5)),I5)))),I5)</f>
+IF($C$1,base!A1,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",A1),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",A1),"$","")=UPPER($C$3),"",I5)),I5))))</f>
         <v>r1</v>
       </c>
       <c r="J5" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="J5" ca="1">IFERROR(IF($C$1,base!B1,
+        <f t="array" aca="1" ref="J5" ca="1">IF($C$1,base!B1,
 IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE)="CASTLE",
 IF(SUBSTITUTE(CELL("address",B1),"$","")=UPPER($A$3),$D$4,
 IF(SUBSTITUTE(CELL("address",B1),"$","")=UPPER($C$3),"",IF(NOT(ISERR(FIND("B",UPPER($A$3)))),
@@ -16838,11 +16363,11 @@
 IF(SUBSTITUTE(CELL("address",B1),"$","")=REPLACE(UPPER($A$3),1,1,"A"),"",J5)),
 IF(SUBSTITUTE(CELL("address",B1),"$","")=REPLACE(UPPER($A$3),1,1,"E"),REPLACE(UPPER($D$4),1,1,"r"),
 IF(SUBSTITUTE(CELL("address",B1),"$","")=REPLACE(UPPER($A$3),1,1,"H"),"",J5))))),
-IF($C$1,base!B1,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",B1),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",B1),"$","")=UPPER($C$3),"",J5)),J5)))),J5)</f>
+IF($C$1,base!B1,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",B1),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",B1),"$","")=UPPER($C$3),"",J5)),J5))))</f>
         <v>n1</v>
       </c>
       <c r="K5" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="K5" ca="1">IFERROR(IF($C$1,base!C1,
+        <f t="array" aca="1" ref="K5" ca="1">IF($C$1,base!C1,
 IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE)="CASTLE",
 IF(SUBSTITUTE(CELL("address",C1),"$","")=UPPER($A$3),$D$4,
 IF(SUBSTITUTE(CELL("address",C1),"$","")=UPPER($C$3),"",IF(NOT(ISERR(FIND("B",UPPER($A$3)))),
@@ -16850,11 +16375,11 @@
 IF(SUBSTITUTE(CELL("address",C1),"$","")=REPLACE(UPPER($A$3),1,1,"A"),"",K5)),
 IF(SUBSTITUTE(CELL("address",C1),"$","")=REPLACE(UPPER($A$3),1,1,"E"),REPLACE(UPPER($D$4),1,1,"r"),
 IF(SUBSTITUTE(CELL("address",C1),"$","")=REPLACE(UPPER($A$3),1,1,"H"),"",K5))))),
-IF($C$1,base!C1,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",C1),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",C1),"$","")=UPPER($C$3),"",K5)),K5)))),K5)</f>
+IF($C$1,base!C1,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",C1),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",C1),"$","")=UPPER($C$3),"",K5)),K5))))</f>
         <v>b1</v>
       </c>
       <c r="L5" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="L5" ca="1">IFERROR(IF($C$1,base!D1,
+        <f t="array" aca="1" ref="L5" ca="1">IF($C$1,base!D1,
 IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE)="CASTLE",
 IF(SUBSTITUTE(CELL("address",D1),"$","")=UPPER($A$3),$D$4,
 IF(SUBSTITUTE(CELL("address",D1),"$","")=UPPER($C$3),"",IF(NOT(ISERR(FIND("B",UPPER($A$3)))),
@@ -16862,11 +16387,11 @@
 IF(SUBSTITUTE(CELL("address",D1),"$","")=REPLACE(UPPER($A$3),1,1,"A"),"",L5)),
 IF(SUBSTITUTE(CELL("address",D1),"$","")=REPLACE(UPPER($A$3),1,1,"E"),REPLACE(UPPER($D$4),1,1,"r"),
 IF(SUBSTITUTE(CELL("address",D1),"$","")=REPLACE(UPPER($A$3),1,1,"H"),"",L5))))),
-IF($C$1,base!D1,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",D1),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",D1),"$","")=UPPER($C$3),"",L5)),L5)))),L5)</f>
+IF($C$1,base!D1,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",D1),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",D1),"$","")=UPPER($C$3),"",L5)),L5))))</f>
         <v>k1</v>
       </c>
       <c r="M5" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="M5" ca="1">IFERROR(IF($C$1,base!E1,
+        <f t="array" aca="1" ref="M5" ca="1">IF($C$1,base!E1,
 IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE)="CASTLE",
 IF(SUBSTITUTE(CELL("address",E1),"$","")=UPPER($A$3),$D$4,
 IF(SUBSTITUTE(CELL("address",E1),"$","")=UPPER($C$3),"",IF(NOT(ISERR(FIND("B",UPPER($A$3)))),
@@ -16874,11 +16399,11 @@
 IF(SUBSTITUTE(CELL("address",E1),"$","")=REPLACE(UPPER($A$3),1,1,"A"),"",M5)),
 IF(SUBSTITUTE(CELL("address",E1),"$","")=REPLACE(UPPER($A$3),1,1,"E"),REPLACE(UPPER($D$4),1,1,"r"),
 IF(SUBSTITUTE(CELL("address",E1),"$","")=REPLACE(UPPER($A$3),1,1,"H"),"",M5))))),
-IF($C$1,base!E1,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",E1),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",E1),"$","")=UPPER($C$3),"",M5)),M5)))),M5)</f>
+IF($C$1,base!E1,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",E1),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",E1),"$","")=UPPER($C$3),"",M5)),M5))))</f>
         <v>q1</v>
       </c>
       <c r="N5" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="N5" ca="1">IFERROR(IF($C$1,base!F1,
+        <f t="array" aca="1" ref="N5" ca="1">IF($C$1,base!F1,
 IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE)="CASTLE",
 IF(SUBSTITUTE(CELL("address",F1),"$","")=UPPER($A$3),$D$4,
 IF(SUBSTITUTE(CELL("address",F1),"$","")=UPPER($C$3),"",IF(NOT(ISERR(FIND("B",UPPER($A$3)))),
@@ -16886,11 +16411,11 @@
 IF(SUBSTITUTE(CELL("address",F1),"$","")=REPLACE(UPPER($A$3),1,1,"A"),"",N5)),
 IF(SUBSTITUTE(CELL("address",F1),"$","")=REPLACE(UPPER($A$3),1,1,"E"),REPLACE(UPPER($D$4),1,1,"r"),
 IF(SUBSTITUTE(CELL("address",F1),"$","")=REPLACE(UPPER($A$3),1,1,"H"),"",N5))))),
-IF($C$1,base!F1,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",F1),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",F1),"$","")=UPPER($C$3),"",N5)),N5)))),N5)</f>
+IF($C$1,base!F1,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",F1),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",F1),"$","")=UPPER($C$3),"",N5)),N5))))</f>
         <v>b1</v>
       </c>
       <c r="O5" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="O5" ca="1">IFERROR(IF($C$1,base!G1,
+        <f t="array" aca="1" ref="O5" ca="1">IF($C$1,base!G1,
 IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE)="CASTLE",
 IF(SUBSTITUTE(CELL("address",G1),"$","")=UPPER($A$3),$D$4,
 IF(SUBSTITUTE(CELL("address",G1),"$","")=UPPER($C$3),"",IF(NOT(ISERR(FIND("B",UPPER($A$3)))),
@@ -16898,11 +16423,11 @@
 IF(SUBSTITUTE(CELL("address",G1),"$","")=REPLACE(UPPER($A$3),1,1,"A"),"",O5)),
 IF(SUBSTITUTE(CELL("address",G1),"$","")=REPLACE(UPPER($A$3),1,1,"E"),REPLACE(UPPER($D$4),1,1,"r"),
 IF(SUBSTITUTE(CELL("address",G1),"$","")=REPLACE(UPPER($A$3),1,1,"H"),"",O5))))),
-IF($C$1,base!G1,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",G1),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",G1),"$","")=UPPER($C$3),"",O5)),O5)))),O5)</f>
+IF($C$1,base!G1,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",G1),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",G1),"$","")=UPPER($C$3),"",O5)),O5))))</f>
         <v>n1</v>
       </c>
       <c r="P5" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="P5" ca="1">IFERROR(IF($C$1,base!H1,
+        <f t="array" aca="1" ref="P5" ca="1">IF($C$1,base!H1,
 IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE)="CASTLE",
 IF(SUBSTITUTE(CELL("address",H1),"$","")=UPPER($A$3),$D$4,
 IF(SUBSTITUTE(CELL("address",H1),"$","")=UPPER($C$3),"",IF(NOT(ISERR(FIND("B",UPPER($A$3)))),
@@ -16910,13 +16435,13 @@
 IF(SUBSTITUTE(CELL("address",H1),"$","")=REPLACE(UPPER($A$3),1,1,"A"),"",P5)),
 IF(SUBSTITUTE(CELL("address",H1),"$","")=REPLACE(UPPER($A$3),1,1,"E"),REPLACE(UPPER($D$4),1,1,"r"),
 IF(SUBSTITUTE(CELL("address",H1),"$","")=REPLACE(UPPER($A$3),1,1,"H"),"",P5))))),
-IF($C$1,base!H1,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",H1),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",H1),"$","")=UPPER($C$3),"",P5)),P5)))),P5)</f>
+IF($C$1,base!H1,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",H1),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",H1),"$","")=UPPER($C$3),"",P5)),P5))))</f>
         <v>r1</v>
       </c>
     </row>
     <row r="6" spans="1:21">
       <c r="I6" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="I6" ca="1">IFERROR(IF($C$1,base!A2,
+        <f t="array" aca="1" ref="I6" ca="1">IF($C$1,base!A2,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",A2),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",A2),"$","")=UPPER($C$3),"",
@@ -16926,11 +16451,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        I6))),
-  I6)),I6)</f>
+  I6))</f>
         <v>p1</v>
       </c>
       <c r="J6" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="J6" ca="1">IFERROR(IF($C$1,base!B2,
+        <f t="array" aca="1" ref="J6" ca="1">IF($C$1,base!B2,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",B2),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",B2),"$","")=UPPER($C$3),"",
@@ -16940,11 +16465,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        J6))),
-  J6)),J6)</f>
+  J6))</f>
         <v>p1</v>
       </c>
       <c r="K6" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="K6" ca="1">IFERROR(IF($C$1,base!C2,
+        <f t="array" aca="1" ref="K6" ca="1">IF($C$1,base!C2,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",C2),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",C2),"$","")=UPPER($C$3),"",
@@ -16954,11 +16479,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        K6))),
-  K6)),K6)</f>
+  K6))</f>
         <v>p1</v>
       </c>
       <c r="L6" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="L6" ca="1">IFERROR(IF($C$1,base!D2,
+        <f t="array" aca="1" ref="L6" ca="1">IF($C$1,base!D2,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",D2),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",D2),"$","")=UPPER($C$3),"",
@@ -16968,11 +16493,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        L6))),
-  L6)),L6)</f>
+  L6))</f>
         <v>p1</v>
       </c>
       <c r="M6" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="M6" ca="1">IFERROR(IF($C$1,base!E2,
+        <f t="array" aca="1" ref="M6" ca="1">IF($C$1,base!E2,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",E2),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",E2),"$","")=UPPER($C$3),"",
@@ -16982,11 +16507,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        M6))),
-  M6)),M6)</f>
+  M6))</f>
         <v>p1</v>
       </c>
       <c r="N6" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="N6" ca="1">IFERROR(IF($C$1,base!F2,
+        <f t="array" aca="1" ref="N6" ca="1">IF($C$1,base!F2,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",F2),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",F2),"$","")=UPPER($C$3),"",
@@ -16996,11 +16521,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        N6))),
-  N6)),N6)</f>
+  N6))</f>
         <v>p1</v>
       </c>
       <c r="O6" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="O6" ca="1">IFERROR(IF($C$1,base!G2,
+        <f t="array" aca="1" ref="O6" ca="1">IF($C$1,base!G2,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",G2),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",G2),"$","")=UPPER($C$3),"",
@@ -17010,11 +16535,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        O6))),
-  O6)),O6)</f>
+  O6))</f>
         <v>p1</v>
       </c>
       <c r="P6" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="P6" ca="1">IFERROR(IF($C$1,base!H2,
+        <f t="array" aca="1" ref="P6" ca="1">IF($C$1,base!H2,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",H2),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",H2),"$","")=UPPER($C$3),"",
@@ -17024,13 +16549,13 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        P6))),
-  P6)),P6)</f>
+  P6))</f>
         <v>p1</v>
       </c>
     </row>
     <row r="7" spans="1:21">
       <c r="I7" s="1" cm="1">
-        <f t="array" aca="1" ref="I7" ca="1">IFERROR(IF($C$1,base!A3,
+        <f t="array" aca="1" ref="I7" ca="1">IF($C$1,base!A3,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",A3),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",A3),"$","")=UPPER($C$3),"",
@@ -17040,11 +16565,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        I7))),
-  I7)),I7)</f>
+  I7))</f>
         <v>0</v>
       </c>
       <c r="J7" s="1" cm="1">
-        <f t="array" aca="1" ref="J7" ca="1">IFERROR(IF($C$1,base!B3,
+        <f t="array" aca="1" ref="J7" ca="1">IF($C$1,base!B3,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",B3),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",B3),"$","")=UPPER($C$3),"",
@@ -17054,11 +16579,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        J7))),
-  J7)),J7)</f>
+  J7))</f>
         <v>0</v>
       </c>
       <c r="K7" s="1" cm="1">
-        <f t="array" aca="1" ref="K7" ca="1">IFERROR(IF($C$1,base!C3,
+        <f t="array" aca="1" ref="K7" ca="1">IF($C$1,base!C3,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",C3),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",C3),"$","")=UPPER($C$3),"",
@@ -17068,11 +16593,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        K7))),
-  K7)),K7)</f>
+  K7))</f>
         <v>0</v>
       </c>
       <c r="L7" s="1" cm="1">
-        <f t="array" aca="1" ref="L7" ca="1">IFERROR(IF($C$1,base!D3,
+        <f t="array" aca="1" ref="L7" ca="1">IF($C$1,base!D3,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",D3),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",D3),"$","")=UPPER($C$3),"",
@@ -17082,11 +16607,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        L7))),
-  L7)),L7)</f>
+  L7))</f>
         <v>0</v>
       </c>
       <c r="M7" s="1" cm="1">
-        <f t="array" aca="1" ref="M7" ca="1">IFERROR(IF($C$1,base!E3,
+        <f t="array" aca="1" ref="M7" ca="1">IF($C$1,base!E3,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",E3),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",E3),"$","")=UPPER($C$3),"",
@@ -17096,11 +16621,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        M7))),
-  M7)),M7)</f>
+  M7))</f>
         <v>0</v>
       </c>
       <c r="N7" s="1" cm="1">
-        <f t="array" aca="1" ref="N7" ca="1">IFERROR(IF($C$1,base!F3,
+        <f t="array" aca="1" ref="N7" ca="1">IF($C$1,base!F3,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",F3),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",F3),"$","")=UPPER($C$3),"",
@@ -17110,11 +16635,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        N7))),
-  N7)),N7)</f>
+  N7))</f>
         <v>0</v>
       </c>
       <c r="O7" s="1" cm="1">
-        <f t="array" aca="1" ref="O7" ca="1">IFERROR(IF($C$1,base!G3,
+        <f t="array" aca="1" ref="O7" ca="1">IF($C$1,base!G3,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",G3),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",G3),"$","")=UPPER($C$3),"",
@@ -17124,11 +16649,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        O7))),
-  O7)),O7)</f>
+  O7))</f>
         <v>0</v>
       </c>
       <c r="P7" s="1" cm="1">
-        <f t="array" aca="1" ref="P7" ca="1">IFERROR(IF($C$1,base!H3,
+        <f t="array" aca="1" ref="P7" ca="1">IF($C$1,base!H3,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",H3),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",H3),"$","")=UPPER($C$3),"",
@@ -17138,13 +16663,13 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        P7))),
-  P7)),P7)</f>
+  P7))</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:21">
       <c r="I8" s="1" cm="1">
-        <f t="array" aca="1" ref="I8" ca="1">IFERROR(IF($C$1,base!A4,
+        <f t="array" aca="1" ref="I8" ca="1">IF($C$1,base!A4,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",A4),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",A4),"$","")=UPPER($C$3),"",
@@ -17154,11 +16679,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        I8))),
-  I8)),I8)</f>
+  I8))</f>
         <v>0</v>
       </c>
       <c r="J8" s="1" cm="1">
-        <f t="array" aca="1" ref="J8" ca="1">IFERROR(IF($C$1,base!B4,
+        <f t="array" aca="1" ref="J8" ca="1">IF($C$1,base!B4,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",B4),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",B4),"$","")=UPPER($C$3),"",
@@ -17168,11 +16693,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        J8))),
-  J8)),J8)</f>
+  J8))</f>
         <v>0</v>
       </c>
       <c r="K8" s="1" cm="1">
-        <f t="array" aca="1" ref="K8" ca="1">IFERROR(IF($C$1,base!C4,
+        <f t="array" aca="1" ref="K8" ca="1">IF($C$1,base!C4,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",C4),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",C4),"$","")=UPPER($C$3),"",
@@ -17182,11 +16707,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        K8))),
-  K8)),K8)</f>
+  K8))</f>
         <v>0</v>
       </c>
       <c r="L8" s="1" cm="1">
-        <f t="array" aca="1" ref="L8" ca="1">IFERROR(IF($C$1,base!D4,
+        <f t="array" aca="1" ref="L8" ca="1">IF($C$1,base!D4,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",D4),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",D4),"$","")=UPPER($C$3),"",
@@ -17196,11 +16721,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        L8))),
-  L8)),L8)</f>
+  L8))</f>
         <v>0</v>
       </c>
       <c r="M8" s="1" cm="1">
-        <f t="array" aca="1" ref="M8" ca="1">IFERROR(IF($C$1,base!E4,
+        <f t="array" aca="1" ref="M8" ca="1">IF($C$1,base!E4,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",E4),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",E4),"$","")=UPPER($C$3),"",
@@ -17210,11 +16735,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        M8))),
-  M8)),M8)</f>
+  M8))</f>
         <v>0</v>
       </c>
       <c r="N8" s="1" cm="1">
-        <f t="array" aca="1" ref="N8" ca="1">IFERROR(IF($C$1,base!F4,
+        <f t="array" aca="1" ref="N8" ca="1">IF($C$1,base!F4,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",F4),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",F4),"$","")=UPPER($C$3),"",
@@ -17224,11 +16749,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        N8))),
-  N8)),N8)</f>
+  N8))</f>
         <v>0</v>
       </c>
       <c r="O8" s="1" cm="1">
-        <f t="array" aca="1" ref="O8" ca="1">IFERROR(IF($C$1,base!G4,
+        <f t="array" aca="1" ref="O8" ca="1">IF($C$1,base!G4,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",G4),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",G4),"$","")=UPPER($C$3),"",
@@ -17238,11 +16763,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        O8))),
-  O8)),O8)</f>
+  O8))</f>
         <v>0</v>
       </c>
       <c r="P8" s="1" cm="1">
-        <f t="array" aca="1" ref="P8" ca="1">IFERROR(IF($C$1,base!H4,
+        <f t="array" aca="1" ref="P8" ca="1">IF($C$1,base!H4,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",H4),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",H4),"$","")=UPPER($C$3),"",
@@ -17252,13 +16777,13 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        P8))),
-  P8)),P8)</f>
+  P8))</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:21" ht="20" customHeight="1">
       <c r="I9" s="1" cm="1">
-        <f t="array" aca="1" ref="I9" ca="1">IFERROR(IF($C$1,base!A5,
+        <f t="array" aca="1" ref="I9" ca="1">IF($C$1,base!A5,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",A5),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",A5),"$","")=UPPER($C$3),"",
@@ -17268,11 +16793,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        I9))),
-  I9)),I9)</f>
+  I9))</f>
         <v>0</v>
       </c>
       <c r="J9" s="1" cm="1">
-        <f t="array" aca="1" ref="J9" ca="1">IFERROR(IF($C$1,base!B5,
+        <f t="array" aca="1" ref="J9" ca="1">IF($C$1,base!B5,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",B5),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",B5),"$","")=UPPER($C$3),"",
@@ -17282,11 +16807,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        J9))),
-  J9)),J9)</f>
+  J9))</f>
         <v>0</v>
       </c>
       <c r="K9" s="1" cm="1">
-        <f t="array" aca="1" ref="K9" ca="1">IFERROR(IF($C$1,base!C5,
+        <f t="array" aca="1" ref="K9" ca="1">IF($C$1,base!C5,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",C5),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",C5),"$","")=UPPER($C$3),"",
@@ -17296,11 +16821,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        K9))),
-  K9)),K9)</f>
+  K9))</f>
         <v>0</v>
       </c>
       <c r="L9" s="1" cm="1">
-        <f t="array" aca="1" ref="L9" ca="1">IFERROR(IF($C$1,base!D5,
+        <f t="array" aca="1" ref="L9" ca="1">IF($C$1,base!D5,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",D5),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",D5),"$","")=UPPER($C$3),"",
@@ -17310,11 +16835,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        L9))),
-  L9)),L9)</f>
+  L9))</f>
         <v>0</v>
       </c>
       <c r="M9" s="1" cm="1">
-        <f t="array" aca="1" ref="M9" ca="1">IFERROR(IF($C$1,base!E5,
+        <f t="array" aca="1" ref="M9" ca="1">IF($C$1,base!E5,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",E5),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",E5),"$","")=UPPER($C$3),"",
@@ -17324,11 +16849,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        M9))),
-  M9)),M9)</f>
+  M9))</f>
         <v>0</v>
       </c>
       <c r="N9" s="1" cm="1">
-        <f t="array" aca="1" ref="N9" ca="1">IFERROR(IF($C$1,base!F5,
+        <f t="array" aca="1" ref="N9" ca="1">IF($C$1,base!F5,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",F5),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",F5),"$","")=UPPER($C$3),"",
@@ -17338,11 +16863,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        N9))),
-  N9)),N9)</f>
+  N9))</f>
         <v>0</v>
       </c>
       <c r="O9" s="1" cm="1">
-        <f t="array" aca="1" ref="O9" ca="1">IFERROR(IF($C$1,base!G5,
+        <f t="array" aca="1" ref="O9" ca="1">IF($C$1,base!G5,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",G5),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",G5),"$","")=UPPER($C$3),"",
@@ -17352,11 +16877,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        O9))),
-  O9)),O9)</f>
+  O9))</f>
         <v>0</v>
       </c>
       <c r="P9" s="1" cm="1">
-        <f t="array" aca="1" ref="P9" ca="1">IFERROR(IF($C$1,base!H5,
+        <f t="array" aca="1" ref="P9" ca="1">IF($C$1,base!H5,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",H5),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",H5),"$","")=UPPER($C$3),"",
@@ -17366,13 +16891,13 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        P9))),
-  P9)),P9)</f>
+  P9))</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:21" ht="20" customHeight="1">
       <c r="I10" s="1" cm="1">
-        <f t="array" aca="1" ref="I10" ca="1">IFERROR(IF($C$1,base!A6,
+        <f t="array" aca="1" ref="I10" ca="1">IF($C$1,base!A6,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",A6),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",A6),"$","")=UPPER($C$3),"",
@@ -17382,11 +16907,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        I10))),
-  I10)),I10)</f>
+  I10))</f>
         <v>0</v>
       </c>
       <c r="J10" s="1" cm="1">
-        <f t="array" aca="1" ref="J10" ca="1">IFERROR(IF($C$1,base!B6,
+        <f t="array" aca="1" ref="J10" ca="1">IF($C$1,base!B6,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",B6),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",B6),"$","")=UPPER($C$3),"",
@@ -17396,11 +16921,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        J10))),
-  J10)),J10)</f>
+  J10))</f>
         <v>0</v>
       </c>
       <c r="K10" s="1" cm="1">
-        <f t="array" aca="1" ref="K10" ca="1">IFERROR(IF($C$1,base!C6,
+        <f t="array" aca="1" ref="K10" ca="1">IF($C$1,base!C6,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",C6),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",C6),"$","")=UPPER($C$3),"",
@@ -17410,11 +16935,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        K10))),
-  K10)),K10)</f>
+  K10))</f>
         <v>0</v>
       </c>
       <c r="L10" s="1" cm="1">
-        <f t="array" aca="1" ref="L10" ca="1">IFERROR(IF($C$1,base!D6,
+        <f t="array" aca="1" ref="L10" ca="1">IF($C$1,base!D6,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",D6),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",D6),"$","")=UPPER($C$3),"",
@@ -17424,11 +16949,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        L10))),
-  L10)),L10)</f>
+  L10))</f>
         <v>0</v>
       </c>
       <c r="M10" s="1" cm="1">
-        <f t="array" aca="1" ref="M10" ca="1">IFERROR(IF($C$1,base!E6,
+        <f t="array" aca="1" ref="M10" ca="1">IF($C$1,base!E6,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",E6),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",E6),"$","")=UPPER($C$3),"",
@@ -17438,11 +16963,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        M10))),
-  M10)),M10)</f>
+  M10))</f>
         <v>0</v>
       </c>
       <c r="N10" s="1" cm="1">
-        <f t="array" aca="1" ref="N10" ca="1">IFERROR(IF($C$1,base!F6,
+        <f t="array" aca="1" ref="N10" ca="1">IF($C$1,base!F6,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",F6),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",F6),"$","")=UPPER($C$3),"",
@@ -17452,11 +16977,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        N10))),
-  N10)),N10)</f>
+  N10))</f>
         <v>0</v>
       </c>
       <c r="O10" s="1" cm="1">
-        <f t="array" aca="1" ref="O10" ca="1">IFERROR(IF($C$1,base!G6,
+        <f t="array" aca="1" ref="O10" ca="1">IF($C$1,base!G6,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",G6),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",G6),"$","")=UPPER($C$3),"",
@@ -17466,11 +16991,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        O10))),
-  O10)),O10)</f>
+  O10))</f>
         <v>0</v>
       </c>
       <c r="P10" s="1" cm="1">
-        <f t="array" aca="1" ref="P10" ca="1">IFERROR(IF($C$1,base!H6,
+        <f t="array" aca="1" ref="P10" ca="1">IF($C$1,base!H6,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",H6),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",H6),"$","")=UPPER($C$3),"",
@@ -17480,13 +17005,13 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        P10))),
-  P10)),P10)</f>
+  P10))</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:21" ht="20" customHeight="1">
       <c r="I11" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="I11" ca="1">IFERROR(IF($C$1,base!A7,
+        <f t="array" aca="1" ref="I11" ca="1">IF($C$1,base!A7,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",A7),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",A7),"$","")=UPPER($C$3),"",
@@ -17496,11 +17021,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        I11))),
-  I11)),I11)</f>
+  I11))</f>
         <v>p2</v>
       </c>
       <c r="J11" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="J11" ca="1">IFERROR(IF($C$1,base!B7,
+        <f t="array" aca="1" ref="J11" ca="1">IF($C$1,base!B7,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",B7),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",B7),"$","")=UPPER($C$3),"",
@@ -17510,11 +17035,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        J11))),
-  J11)),J11)</f>
+  J11))</f>
         <v>p2</v>
       </c>
       <c r="K11" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="K11" ca="1">IFERROR(IF($C$1,base!C7,
+        <f t="array" aca="1" ref="K11" ca="1">IF($C$1,base!C7,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",C7),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",C7),"$","")=UPPER($C$3),"",
@@ -17524,11 +17049,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        K11))),
-  K11)),K11)</f>
+  K11))</f>
         <v>p2</v>
       </c>
       <c r="L11" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="L11" ca="1">IFERROR(IF($C$1,base!D7,
+        <f t="array" aca="1" ref="L11" ca="1">IF($C$1,base!D7,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",D7),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",D7),"$","")=UPPER($C$3),"",
@@ -17538,11 +17063,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        L11))),
-  L11)),L11)</f>
+  L11))</f>
         <v>p2</v>
       </c>
       <c r="M11" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="M11" ca="1">IFERROR(IF($C$1,base!E7,
+        <f t="array" aca="1" ref="M11" ca="1">IF($C$1,base!E7,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",E7),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",E7),"$","")=UPPER($C$3),"",
@@ -17552,11 +17077,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        M11))),
-  M11)),M11)</f>
+  M11))</f>
         <v>p2</v>
       </c>
       <c r="N11" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="N11" ca="1">IFERROR(IF($C$1,base!F7,
+        <f t="array" aca="1" ref="N11" ca="1">IF($C$1,base!F7,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",F7),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",F7),"$","")=UPPER($C$3),"",
@@ -17566,11 +17091,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        N11))),
-  N11)),N11)</f>
+  N11))</f>
         <v>p2</v>
       </c>
       <c r="O11" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="O11" ca="1">IFERROR(IF($C$1,base!G7,
+        <f t="array" aca="1" ref="O11" ca="1">IF($C$1,base!G7,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",G7),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",G7),"$","")=UPPER($C$3),"",
@@ -17580,11 +17105,11 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        O11))),
-  O11)),O11)</f>
+  O11))</f>
         <v>p2</v>
       </c>
       <c r="P11" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="P11" ca="1">IFERROR(IF($C$1,base!H7,
+        <f t="array" aca="1" ref="P11" ca="1">IF($C$1,base!H7,
  IF(($B$4=TRUE),
   IF(SUBSTITUTE(CELL("address",H7),"$","")=UPPER($A$3),$D$4,
    IF(SUBSTITUTE(CELL("address",H7),"$","")=UPPER($C$3),"",
@@ -17594,13 +17119,13 @@
            OR(inputsimplified!$K$10="",inputsimplified!$K$10=0)),
        "",
        P11))),
-  P11)),P11)</f>
+  P11))</f>
         <v>p2</v>
       </c>
     </row>
     <row r="12" spans="1:21" ht="20" customHeight="1">
       <c r="I12" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="I12" ca="1">IFERROR(IF($C$1,base!A8,
+        <f t="array" aca="1" ref="I12" ca="1">IF($C$1,base!A8,
 IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE)="CASTLE",
 IF(SUBSTITUTE(CELL("address",A8),"$","")=UPPER($A$3),$D$4,
 IF(SUBSTITUTE(CELL("address",A8),"$","")=UPPER($C$3),"",IF(NOT(ISERR(FIND("B",UPPER($A$3)))),
@@ -17608,11 +17133,11 @@
 IF(SUBSTITUTE(CELL("address",A8),"$","")=REPLACE(UPPER($A$3),1,1,"A"),"",I12)),
 IF(SUBSTITUTE(CELL("address",A8),"$","")=REPLACE(UPPER($A$3),1,1,"E"),REPLACE(UPPER($D$4),1,1,"r"),
 IF(SUBSTITUTE(CELL("address",A8),"$","")=REPLACE(UPPER($A$3),1,1,"H"),"",I12))))),
-IF($C$1,base!A8,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",A8),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",A8),"$","")=UPPER($C$3),"",I12)),I12)))),I12)</f>
+IF($C$1,base!A8,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",A8),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",A8),"$","")=UPPER($C$3),"",I12)),I12))))</f>
         <v>r2</v>
       </c>
       <c r="J12" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="J12" ca="1">IFERROR(IF($C$1,base!B8,
+        <f t="array" aca="1" ref="J12" ca="1">IF($C$1,base!B8,
 IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE)="CASTLE",
 IF(SUBSTITUTE(CELL("address",B8),"$","")=UPPER($A$3),$D$4,
 IF(SUBSTITUTE(CELL("address",B8),"$","")=UPPER($C$3),"",IF(NOT(ISERR(FIND("B",UPPER($A$3)))),
@@ -17620,11 +17145,11 @@
 IF(SUBSTITUTE(CELL("address",B8),"$","")=REPLACE(UPPER($A$3),1,1,"A"),"",J12)),
 IF(SUBSTITUTE(CELL("address",B8),"$","")=REPLACE(UPPER($A$3),1,1,"E"),REPLACE(UPPER($D$4),1,1,"r"),
 IF(SUBSTITUTE(CELL("address",B8),"$","")=REPLACE(UPPER($A$3),1,1,"H"),"",J12))))),
-IF($C$1,base!B8,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",B8),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",B8),"$","")=UPPER($C$3),"",J12)),J12)))),J12)</f>
+IF($C$1,base!B8,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",B8),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",B8),"$","")=UPPER($C$3),"",J12)),J12))))</f>
         <v>n2</v>
       </c>
       <c r="K12" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="K12" ca="1">IFERROR(IF($C$1,base!C8,
+        <f t="array" aca="1" ref="K12" ca="1">IF($C$1,base!C8,
 IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE)="CASTLE",
 IF(SUBSTITUTE(CELL("address",C8),"$","")=UPPER($A$3),$D$4,
 IF(SUBSTITUTE(CELL("address",C8),"$","")=UPPER($C$3),"",IF(NOT(ISERR(FIND("B",UPPER($A$3)))),
@@ -17632,11 +17157,11 @@
 IF(SUBSTITUTE(CELL("address",C8),"$","")=REPLACE(UPPER($A$3),1,1,"A"),"",K12)),
 IF(SUBSTITUTE(CELL("address",C8),"$","")=REPLACE(UPPER($A$3),1,1,"E"),REPLACE(UPPER($D$4),1,1,"r"),
 IF(SUBSTITUTE(CELL("address",C8),"$","")=REPLACE(UPPER($A$3),1,1,"H"),"",K12))))),
-IF($C$1,base!C8,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",C8),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",C8),"$","")=UPPER($C$3),"",K12)),K12)))),K12)</f>
+IF($C$1,base!C8,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",C8),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",C8),"$","")=UPPER($C$3),"",K12)),K12))))</f>
         <v>b2</v>
       </c>
       <c r="L12" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="L12" ca="1">IFERROR(IF($C$1,base!D8,
+        <f t="array" aca="1" ref="L12" ca="1">IF($C$1,base!D8,
 IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE)="CASTLE",
 IF(SUBSTITUTE(CELL("address",D8),"$","")=UPPER($A$3),$D$4,
 IF(SUBSTITUTE(CELL("address",D8),"$","")=UPPER($C$3),"",IF(NOT(ISERR(FIND("B",UPPER($A$3)))),
@@ -17644,11 +17169,11 @@
 IF(SUBSTITUTE(CELL("address",D8),"$","")=REPLACE(UPPER($A$3),1,1,"A"),"",L12)),
 IF(SUBSTITUTE(CELL("address",D8),"$","")=REPLACE(UPPER($A$3),1,1,"E"),REPLACE(UPPER($D$4),1,1,"r"),
 IF(SUBSTITUTE(CELL("address",D8),"$","")=REPLACE(UPPER($A$3),1,1,"H"),"",L12))))),
-IF($C$1,base!D8,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",D8),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",D8),"$","")=UPPER($C$3),"",L12)),L12)))),L12)</f>
+IF($C$1,base!D8,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",D8),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",D8),"$","")=UPPER($C$3),"",L12)),L12))))</f>
         <v>k2</v>
       </c>
       <c r="M12" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="M12" ca="1">IFERROR(IF($C$1,base!E8,
+        <f t="array" aca="1" ref="M12" ca="1">IF($C$1,base!E8,
 IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE)="CASTLE",
 IF(SUBSTITUTE(CELL("address",E8),"$","")=UPPER($A$3),$D$4,
 IF(SUBSTITUTE(CELL("address",E8),"$","")=UPPER($C$3),"",IF(NOT(ISERR(FIND("B",UPPER($A$3)))),
@@ -17656,11 +17181,11 @@
 IF(SUBSTITUTE(CELL("address",E8),"$","")=REPLACE(UPPER($A$3),1,1,"A"),"",M12)),
 IF(SUBSTITUTE(CELL("address",E8),"$","")=REPLACE(UPPER($A$3),1,1,"E"),REPLACE(UPPER($D$4),1,1,"r"),
 IF(SUBSTITUTE(CELL("address",E8),"$","")=REPLACE(UPPER($A$3),1,1,"H"),"",M12))))),
-IF($C$1,base!E8,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",E8),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",E8),"$","")=UPPER($C$3),"",M12)),M12)))),M12)</f>
+IF($C$1,base!E8,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",E8),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",E8),"$","")=UPPER($C$3),"",M12)),M12))))</f>
         <v>q2</v>
       </c>
       <c r="N12" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="N12" ca="1">IFERROR(IF($C$1,base!F8,
+        <f t="array" aca="1" ref="N12" ca="1">IF($C$1,base!F8,
 IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE)="CASTLE",
 IF(SUBSTITUTE(CELL("address",F8),"$","")=UPPER($A$3),$D$4,
 IF(SUBSTITUTE(CELL("address",F8),"$","")=UPPER($C$3),"",IF(NOT(ISERR(FIND("B",UPPER($A$3)))),
@@ -17668,11 +17193,11 @@
 IF(SUBSTITUTE(CELL("address",F8),"$","")=REPLACE(UPPER($A$3),1,1,"A"),"",N12)),
 IF(SUBSTITUTE(CELL("address",F8),"$","")=REPLACE(UPPER($A$3),1,1,"E"),REPLACE(UPPER($D$4),1,1,"r"),
 IF(SUBSTITUTE(CELL("address",F8),"$","")=REPLACE(UPPER($A$3),1,1,"H"),"",N12))))),
-IF($C$1,base!F8,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",F8),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",F8),"$","")=UPPER($C$3),"",N12)),N12)))),N12)</f>
+IF($C$1,base!F8,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",F8),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",F8),"$","")=UPPER($C$3),"",N12)),N12))))</f>
         <v>b2</v>
       </c>
       <c r="O12" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="O12" ca="1">IFERROR(IF($C$1,base!G8,
+        <f t="array" aca="1" ref="O12" ca="1">IF($C$1,base!G8,
 IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE)="CASTLE",
 IF(SUBSTITUTE(CELL("address",G8),"$","")=UPPER($A$3),$D$4,
 IF(SUBSTITUTE(CELL("address",G8),"$","")=UPPER($C$3),"",IF(NOT(ISERR(FIND("B",UPPER($A$3)))),
@@ -17680,11 +17205,11 @@
 IF(SUBSTITUTE(CELL("address",G8),"$","")=REPLACE(UPPER($A$3),1,1,"A"),"",O12)),
 IF(SUBSTITUTE(CELL("address",G8),"$","")=REPLACE(UPPER($A$3),1,1,"E"),REPLACE(UPPER($D$4),1,1,"r"),
 IF(SUBSTITUTE(CELL("address",G8),"$","")=REPLACE(UPPER($A$3),1,1,"H"),"",O12))))),
-IF($C$1,base!G8,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",G8),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",G8),"$","")=UPPER($C$3),"",O12)),O12)))),O12)</f>
+IF($C$1,base!G8,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",G8),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",G8),"$","")=UPPER($C$3),"",O12)),O12))))</f>
         <v>n2</v>
       </c>
       <c r="P12" s="1" t="str" cm="1">
-        <f t="array" aca="1" ref="P12" ca="1">IFERROR(IF($C$1,base!H8,
+        <f t="array" aca="1" ref="P12" ca="1">IF($C$1,base!H8,
 IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE)="CASTLE",
 IF(SUBSTITUTE(CELL("address",H8),"$","")=UPPER($A$3),$D$4,
 IF(SUBSTITUTE(CELL("address",H8),"$","")=UPPER($C$3),"",IF(NOT(ISERR(FIND("B",UPPER($A$3)))),
@@ -17692,7 +17217,7 @@
 IF(SUBSTITUTE(CELL("address",H8),"$","")=REPLACE(UPPER($A$3),1,1,"A"),"",P12)),
 IF(SUBSTITUTE(CELL("address",H8),"$","")=REPLACE(UPPER($A$3),1,1,"E"),REPLACE(UPPER($D$4),1,1,"r"),
 IF(SUBSTITUTE(CELL("address",H8),"$","")=REPLACE(UPPER($A$3),1,1,"H"),"",P12))))),
-IF($C$1,base!H8,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",H8),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",H8),"$","")=UPPER($C$3),"",P12)),P12)))),P12)</f>
+IF($C$1,base!H8,IF(IFERROR(_xlfn.IFNA($B$4,FALSE),FALSE),IF(SUBSTITUTE(CELL("address",H8),"$","")=UPPER($A$3),SUBSTITUTE($D$4,"p","q"),IF(SUBSTITUTE(CELL("address",H8),"$","")=UPPER($C$3),"",P12)),P12))))</f>
         <v>r2</v>
       </c>
     </row>
@@ -35604,608 +35129,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheetPr>
-    <tabColor rgb="FF6B6B6B"/>
-  </sheetPr>
-  <dimension ref="A1:N26"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
-  <cols>
-    <col min="1" max="1" width="30" customWidth="1"/>
-    <col min="2" max="6" width="6" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="9" width="6" customWidth="1"/>
-    <col min="10" max="10" width="3" customWidth="1"/>
-    <col min="11" max="11" width="24" customWidth="1"/>
-    <col min="12" max="12" width="40" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CHESS ENGINE  /  working sheet</t>
-        </is>
-      </c>
-      <c r="K1" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Side to move</t>
-        </is>
-      </c>
-      <c r="L1" s="38">
-        <f ca="1">livegame!R16</f>
-      </c>
-      <c r="M1" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Engine plays</t>
-        </is>
-      </c>
-      <c r="N1" s="38">
-        <f ca="1">IFERROR(UPPER(Coach!$C$20),"OFF")</f>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nothing here needs touching. Read the Coach tab instead.</t>
-        </is>
-      </c>
-      <c r="K2" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Colour</t>
-        </is>
-      </c>
-      <c r="L2" s="38">
-        <f ca="1">IF(L1=1,"White","Black")</f>
-      </c>
-      <c r="M2" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bot side (1=W 2=B)</t>
-        </is>
-      </c>
-      <c r="N2" s="38">
-        <f ca="1">IF($N$1="BLACK",2,IF($N$1="WHITE",1,0))</f>
-      </c>
-    </row>
-    <row r="3">
-      <c r="K3" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Engine on</t>
-        </is>
-      </c>
-      <c r="L3" s="38">
-        <f ca="1">OR(UPPER(Coach!$C$18)="ON",Coach!$C$18="")</f>
-      </c>
-      <c r="M3" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">from</t>
-        </is>
-      </c>
-      <c r="N3" s="38">
-        <f ca="1">IFERROR(IF($N$9=0,"",xSQ($N$9,$N$10)),"")</f>
-      </c>
-    </row>
-    <row r="4">
-      <c r="K4" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Candidates kept</t>
-        </is>
-      </c>
-      <c r="L4" s="38">
-        <f ca="1">IFERROR(MAX(2,MIN(16,VALUE(Coach!$C$19))),8)</f>
-      </c>
-      <c r="M4" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to</t>
-        </is>
-      </c>
-      <c r="N4" s="38">
-        <f ca="1">IFERROR(IF($N$11=0,"",xSQ($N$11,$N$12)),"")</f>
-      </c>
-    </row>
-    <row r="5">
-      <c r="M5" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">piece</t>
-        </is>
-      </c>
-      <c r="N5" s="38">
-        <f ca="1">IFERROR(IF($N$9=0,"",INDEX($B$10:$I$17,$N$9,$N$10)),"")</f>
-      </c>
-    </row>
-    <row r="6">
-      <c r="K6" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Stage 1  candidate list</t>
-        </is>
-      </c>
-      <c r="L6" s="38">
-        <f ca="1">_xlfn.LET(_xlpm.on,$L$3,_xlpm.n,$L$4,_xlpm.bd,$B$10:$I$17,_xlpm.sd,TEXT($L$1,"0"),IF(NOT(_xlpm.on),"",_xlfn.LET(_xlpm.g,xGEN(_xlpm.bd,_xlpm.sd),_xlpm.ky,_xlfn.CHOOSECOLS(_xlpm.g,1),_xlpm.nm,ROWS(_xlpm.ky)-1,_xlfn.REDUCE("",_xlfn.SEQUENCE(_xlpm.n),_xlfn.LAMBDA(_xlpm.a,_xlpm.k,IF(_xlpm.k&gt;_xlpm.nm,_xlpm.a,_xlfn.LET(_xlpm.v,LARGE(_xlpm.ky,_xlpm.k),IF(_xlpm.v&lt;=-900000000,_xlpm.a,_xlfn.LET(_xlpm.i,MATCH(_xlpm.v,_xlpm.ky,0),_xlpm.a&amp;INDEX(_xlpm.g,_xlpm.i,3)&amp;INDEX(_xlpm.g,_xlpm.i,4)&amp;INDEX(_xlpm.g,_xlpm.i,5)&amp;INDEX(_xlpm.g,_xlpm.i,6))))))))))</f>
-      </c>
-      <c r="M6" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bot to move now</t>
-        </is>
-      </c>
-      <c r="N6" s="38">
-        <f ca="1">IFERROR(AND($N$2&gt;0,livegame!$R$16=$N$2,$L$1=$N$2,RIGHT($N$5,1)=TEXT($N$2,"0"),livegame!$C$1&lt;&gt;TRUE,livegame!$S$17="",$N$3&lt;&gt;"",$N$4&lt;&gt;"",$N$5&lt;&gt;"",Sheet1!$BH$1),FALSE)</f>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Board mirror of livegame!I5:P12</t>
-        </is>
-      </c>
-      <c r="K7" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Stage 2  2-ply ranked</t>
-        </is>
-      </c>
-      <c r="L7" s="38">
-        <f ca="1">IF($L$1=$N$2,"",_xlfn.LET(_xlpm.s,$L$6,_xlpm.bd,$B$10:$I$17,_xlpm.sd,TEXT($L$1,"0"),_xlpm.et,IF(_xlpm.sd="1","2","1"),_xlpm.sg,IF(_xlpm.sd="1",1,-1),_xlpm.n,INT(LEN(_xlpm.s)/4),IF(_xlpm.n=0,"",_xlfn.LET(_xlpm.rc,_xlfn.REDUCE("",_xlfn.SEQUENCE(_xlpm.n),_xlfn.LAMBDA(_xlpm.a,_xlpm.k,_xlfn.LET(_xlpm.fr,VALUE(MID(_xlpm.s,(_xlpm.k-1)*4+1,1)),_xlpm.fc,VALUE(MID(_xlpm.s,(_xlpm.k-1)*4+2,1)),_xlpm.tr,VALUE(MID(_xlpm.s,(_xlpm.k-1)*4+3,1)),_xlpm.tc,VALUE(MID(_xlpm.s,(_xlpm.k-1)*4+4,1)),_xlpm.hd,_xlpm.fr&amp;_xlpm.fc&amp;_xlpm.tr&amp;_xlpm.tc,_xlpm.sm,xSIM(_xlpm.bd,_xlpm.fr,_xlpm.fc,_xlpm.tr,_xlpm.tc),_xlpm.ek,xKLOC(_xlpm.sm,_xlpm.et),IF(_xlpm.ek=0,_xlpm.a&amp;_xlpm.hd&amp;"100"&amp;TEXT(700000,"0000000"),_xlfn.LET(_xlpm.ch,IF(xATT(_xlpm.sm,INT(_xlpm.ek/10),MOD(_xlpm.ek,10),_xlpm.sd),1,0),_xlpm.g,xGEN(_xlpm.sm,_xlpm.et),IF(ROWS(_xlpm.g)=1,_xlpm.a&amp;_xlpm.hd&amp;_xlpm.ch&amp;IF(_xlpm.ch=1,"10","01")&amp;TEXT(IF(_xlpm.ch=1,600000,500000),"0000000"),_xlfn.LET(_xlpm.gg,_xlfn.DROP(_xlpm.g,1),_xlpm.s2,MIN(_xlpm.sg*_xlfn.CHOOSECOLS(_xlpm.gg,8)+_xlfn.CHOOSECOLS(_xlpm.gg,7)),_xlpm.a&amp;_xlpm.hd&amp;_xlpm.ch&amp;"00"&amp;TEXT(ROUND(_xlpm.s2,0)+500000,"0000000")))))))),_xlpm.ar,_xlfn.MAKEARRAY(_xlpm.n,1,_xlfn.LAMBDA(_xlpm.k,_xlpm.c,VALUE(MID(_xlpm.rc,(_xlpm.k-1)*14+8,7))*100+(_xlpm.n-_xlpm.k))),_xlfn.REDUCE("",_xlfn.SEQUENCE(MIN(6,_xlpm.n)),_xlfn.LAMBDA(_xlpm.a,_xlpm.k,_xlfn.LET(_xlpm.v,LARGE(_xlpm.ar,_xlpm.k),_xlpm.i,MATCH(_xlpm.v,_xlpm.ar,0),_xlpm.a&amp;MID(_xlpm.rc,(_xlpm.i-1)*14+1,14))))))))</f>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">row 1 = White back rank, col 1 = file A</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="N9" s="38">
-        <f ca="1">IFERROR(IF(LEN($L$6)&lt;4,0,VALUE(MID($L$6,1,1))),0)</f>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="48">
-        <f ca="1">IF(OR(livegame!I5="",livegame!I5=0),"",livegame!I5&amp;"")</f>
-      </c>
-      <c r="C10" s="48">
-        <f ca="1">IF(OR(livegame!J5="",livegame!J5=0),"",livegame!J5&amp;"")</f>
-      </c>
-      <c r="D10" s="48">
-        <f ca="1">IF(OR(livegame!K5="",livegame!K5=0),"",livegame!K5&amp;"")</f>
-      </c>
-      <c r="E10" s="48">
-        <f ca="1">IF(OR(livegame!L5="",livegame!L5=0),"",livegame!L5&amp;"")</f>
-      </c>
-      <c r="F10" s="48">
-        <f ca="1">IF(OR(livegame!M5="",livegame!M5=0),"",livegame!M5&amp;"")</f>
-      </c>
-      <c r="G10" s="48">
-        <f ca="1">IF(OR(livegame!N5="",livegame!N5=0),"",livegame!N5&amp;"")</f>
-      </c>
-      <c r="H10" s="48">
-        <f ca="1">IF(OR(livegame!O5="",livegame!O5=0),"",livegame!O5&amp;"")</f>
-      </c>
-      <c r="I10" s="48">
-        <f ca="1">IF(OR(livegame!P5="",livegame!P5=0),"",livegame!P5&amp;"")</f>
-      </c>
-      <c r="N10" s="38">
-        <f ca="1">IFERROR(IF(LEN($L$6)&lt;4,0,VALUE(MID($L$6,2,1))),0)</f>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="48">
-        <f ca="1">IF(OR(livegame!I6="",livegame!I6=0),"",livegame!I6&amp;"")</f>
-      </c>
-      <c r="C11" s="48">
-        <f ca="1">IF(OR(livegame!J6="",livegame!J6=0),"",livegame!J6&amp;"")</f>
-      </c>
-      <c r="D11" s="48">
-        <f ca="1">IF(OR(livegame!K6="",livegame!K6=0),"",livegame!K6&amp;"")</f>
-      </c>
-      <c r="E11" s="48">
-        <f ca="1">IF(OR(livegame!L6="",livegame!L6=0),"",livegame!L6&amp;"")</f>
-      </c>
-      <c r="F11" s="48">
-        <f ca="1">IF(OR(livegame!M6="",livegame!M6=0),"",livegame!M6&amp;"")</f>
-      </c>
-      <c r="G11" s="48">
-        <f ca="1">IF(OR(livegame!N6="",livegame!N6=0),"",livegame!N6&amp;"")</f>
-      </c>
-      <c r="H11" s="48">
-        <f ca="1">IF(OR(livegame!O6="",livegame!O6=0),"",livegame!O6&amp;"")</f>
-      </c>
-      <c r="I11" s="48">
-        <f ca="1">IF(OR(livegame!P6="",livegame!P6=0),"",livegame!P6&amp;"")</f>
-      </c>
-      <c r="N11" s="38">
-        <f ca="1">IFERROR(IF(LEN($L$6)&lt;4,0,VALUE(MID($L$6,3,1))),0)</f>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" s="48">
-        <f ca="1">IF(OR(livegame!I7="",livegame!I7=0),"",livegame!I7&amp;"")</f>
-      </c>
-      <c r="C12" s="48">
-        <f ca="1">IF(OR(livegame!J7="",livegame!J7=0),"",livegame!J7&amp;"")</f>
-      </c>
-      <c r="D12" s="48">
-        <f ca="1">IF(OR(livegame!K7="",livegame!K7=0),"",livegame!K7&amp;"")</f>
-      </c>
-      <c r="E12" s="48">
-        <f ca="1">IF(OR(livegame!L7="",livegame!L7=0),"",livegame!L7&amp;"")</f>
-      </c>
-      <c r="F12" s="48">
-        <f ca="1">IF(OR(livegame!M7="",livegame!M7=0),"",livegame!M7&amp;"")</f>
-      </c>
-      <c r="G12" s="48">
-        <f ca="1">IF(OR(livegame!N7="",livegame!N7=0),"",livegame!N7&amp;"")</f>
-      </c>
-      <c r="H12" s="48">
-        <f ca="1">IF(OR(livegame!O7="",livegame!O7=0),"",livegame!O7&amp;"")</f>
-      </c>
-      <c r="I12" s="48">
-        <f ca="1">IF(OR(livegame!P7="",livegame!P7=0),"",livegame!P7&amp;"")</f>
-      </c>
-      <c r="N12" s="38">
-        <f ca="1">IFERROR(IF(LEN($L$6)&lt;4,0,VALUE(MID($L$6,4,1))),0)</f>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="48">
-        <f ca="1">IF(OR(livegame!I8="",livegame!I8=0),"",livegame!I8&amp;"")</f>
-      </c>
-      <c r="C13" s="48">
-        <f ca="1">IF(OR(livegame!J8="",livegame!J8=0),"",livegame!J8&amp;"")</f>
-      </c>
-      <c r="D13" s="48">
-        <f ca="1">IF(OR(livegame!K8="",livegame!K8=0),"",livegame!K8&amp;"")</f>
-      </c>
-      <c r="E13" s="48">
-        <f ca="1">IF(OR(livegame!L8="",livegame!L8=0),"",livegame!L8&amp;"")</f>
-      </c>
-      <c r="F13" s="48">
-        <f ca="1">IF(OR(livegame!M8="",livegame!M8=0),"",livegame!M8&amp;"")</f>
-      </c>
-      <c r="G13" s="48">
-        <f ca="1">IF(OR(livegame!N8="",livegame!N8=0),"",livegame!N8&amp;"")</f>
-      </c>
-      <c r="H13" s="48">
-        <f ca="1">IF(OR(livegame!O8="",livegame!O8=0),"",livegame!O8&amp;"")</f>
-      </c>
-      <c r="I13" s="48">
-        <f ca="1">IF(OR(livegame!P8="",livegame!P8=0),"",livegame!P8&amp;"")</f>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="48">
-        <f ca="1">IF(OR(livegame!I9="",livegame!I9=0),"",livegame!I9&amp;"")</f>
-      </c>
-      <c r="C14" s="48">
-        <f ca="1">IF(OR(livegame!J9="",livegame!J9=0),"",livegame!J9&amp;"")</f>
-      </c>
-      <c r="D14" s="48">
-        <f ca="1">IF(OR(livegame!K9="",livegame!K9=0),"",livegame!K9&amp;"")</f>
-      </c>
-      <c r="E14" s="48">
-        <f ca="1">IF(OR(livegame!L9="",livegame!L9=0),"",livegame!L9&amp;"")</f>
-      </c>
-      <c r="F14" s="48">
-        <f ca="1">IF(OR(livegame!M9="",livegame!M9=0),"",livegame!M9&amp;"")</f>
-      </c>
-      <c r="G14" s="48">
-        <f ca="1">IF(OR(livegame!N9="",livegame!N9=0),"",livegame!N9&amp;"")</f>
-      </c>
-      <c r="H14" s="48">
-        <f ca="1">IF(OR(livegame!O9="",livegame!O9=0),"",livegame!O9&amp;"")</f>
-      </c>
-      <c r="I14" s="48">
-        <f ca="1">IF(OR(livegame!P9="",livegame!P9=0),"",livegame!P9&amp;"")</f>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="48">
-        <f ca="1">IF(OR(livegame!I10="",livegame!I10=0),"",livegame!I10&amp;"")</f>
-      </c>
-      <c r="C15" s="48">
-        <f ca="1">IF(OR(livegame!J10="",livegame!J10=0),"",livegame!J10&amp;"")</f>
-      </c>
-      <c r="D15" s="48">
-        <f ca="1">IF(OR(livegame!K10="",livegame!K10=0),"",livegame!K10&amp;"")</f>
-      </c>
-      <c r="E15" s="48">
-        <f ca="1">IF(OR(livegame!L10="",livegame!L10=0),"",livegame!L10&amp;"")</f>
-      </c>
-      <c r="F15" s="48">
-        <f ca="1">IF(OR(livegame!M10="",livegame!M10=0),"",livegame!M10&amp;"")</f>
-      </c>
-      <c r="G15" s="48">
-        <f ca="1">IF(OR(livegame!N10="",livegame!N10=0),"",livegame!N10&amp;"")</f>
-      </c>
-      <c r="H15" s="48">
-        <f ca="1">IF(OR(livegame!O10="",livegame!O10=0),"",livegame!O10&amp;"")</f>
-      </c>
-      <c r="I15" s="48">
-        <f ca="1">IF(OR(livegame!P10="",livegame!P10=0),"",livegame!P10&amp;"")</f>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="48">
-        <f ca="1">IF(OR(livegame!I11="",livegame!I11=0),"",livegame!I11&amp;"")</f>
-      </c>
-      <c r="C16" s="48">
-        <f ca="1">IF(OR(livegame!J11="",livegame!J11=0),"",livegame!J11&amp;"")</f>
-      </c>
-      <c r="D16" s="48">
-        <f ca="1">IF(OR(livegame!K11="",livegame!K11=0),"",livegame!K11&amp;"")</f>
-      </c>
-      <c r="E16" s="48">
-        <f ca="1">IF(OR(livegame!L11="",livegame!L11=0),"",livegame!L11&amp;"")</f>
-      </c>
-      <c r="F16" s="48">
-        <f ca="1">IF(OR(livegame!M11="",livegame!M11=0),"",livegame!M11&amp;"")</f>
-      </c>
-      <c r="G16" s="48">
-        <f ca="1">IF(OR(livegame!N11="",livegame!N11=0),"",livegame!N11&amp;"")</f>
-      </c>
-      <c r="H16" s="48">
-        <f ca="1">IF(OR(livegame!O11="",livegame!O11=0),"",livegame!O11&amp;"")</f>
-      </c>
-      <c r="I16" s="48">
-        <f ca="1">IF(OR(livegame!P11="",livegame!P11=0),"",livegame!P11&amp;"")</f>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="48">
-        <f ca="1">IF(OR(livegame!I12="",livegame!I12=0),"",livegame!I12&amp;"")</f>
-      </c>
-      <c r="C17" s="48">
-        <f ca="1">IF(OR(livegame!J12="",livegame!J12=0),"",livegame!J12&amp;"")</f>
-      </c>
-      <c r="D17" s="48">
-        <f ca="1">IF(OR(livegame!K12="",livegame!K12=0),"",livegame!K12&amp;"")</f>
-      </c>
-      <c r="E17" s="48">
-        <f ca="1">IF(OR(livegame!L12="",livegame!L12=0),"",livegame!L12&amp;"")</f>
-      </c>
-      <c r="F17" s="48">
-        <f ca="1">IF(OR(livegame!M12="",livegame!M12=0),"",livegame!M12&amp;"")</f>
-      </c>
-      <c r="G17" s="48">
-        <f ca="1">IF(OR(livegame!N12="",livegame!N12=0),"",livegame!N12&amp;"")</f>
-      </c>
-      <c r="H17" s="48">
-        <f ca="1">IF(OR(livegame!O12="",livegame!O12=0),"",livegame!O12&amp;"")</f>
-      </c>
-      <c r="I17" s="48">
-        <f ca="1">IF(OR(livegame!P12="",livegame!P12=0),"",livegame!P12&amp;"")</f>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ranked moves</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">#</t>
-        </is>
-      </c>
-      <c r="B20" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">record</t>
-        </is>
-      </c>
-      <c r="C20" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">from</t>
-        </is>
-      </c>
-      <c r="D20" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">to</t>
-        </is>
-      </c>
-      <c r="E20" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">piece</t>
-        </is>
-      </c>
-      <c r="F20" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">glyph</t>
-        </is>
-      </c>
-      <c r="G20" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">eval</t>
-        </is>
-      </c>
-      <c r="H20" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">type</t>
-        </is>
-      </c>
-      <c r="I20" s="37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">why</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="38">
-        <v>1</v>
-      </c>
-      <c r="B21" s="38">
-        <f ca="1">IF(LEN($L$7)&gt;=$A21*14,MID($L$7,($A21-1)*14+1,14),"")</f>
-      </c>
-      <c r="C21" s="38">
-        <f ca="1">IF($B21="","",xSQ(VALUE(MID($B21,1,1)),VALUE(MID($B21,2,1))))</f>
-      </c>
-      <c r="D21" s="38">
-        <f ca="1">IF($B21="","",xSQ(VALUE(MID($B21,3,1)),VALUE(MID($B21,4,1))))</f>
-      </c>
-      <c r="E21" s="38">
-        <f ca="1">IF($B21="","",xPN(INDEX($B$10:$I$17,VALUE(MID($B21,1,1)),VALUE(MID($B21,2,1)))))</f>
-      </c>
-      <c r="F21" s="38">
-        <f ca="1">IF($B21="","",xGLY(INDEX($B$10:$I$17,VALUE(MID($B21,1,1)),VALUE(MID($B21,2,1)))))</f>
-      </c>
-      <c r="G21" s="44">
-        <f ca="1">IF($B21="","",(VALUE(MID($B21,8,7))-500000)/100)</f>
-      </c>
-      <c r="H21" s="38">
-        <f ca="1">IF($B21="","",IF(MID($B21,6,1)="1","Checkmate",IF(MID($B21,7,1)="1","Stalemate",IF(MID($B21,5,1)="1","Check",IF(INDEX($B$10:$I$17,VALUE(MID($B21,3,1)),VALUE(MID($B21,4,1)))&lt;&gt;"","Capture","Quiet")))))</f>
-      </c>
-      <c r="I21" s="38">
-        <f ca="1">IF($B21="","",_xlfn.LET(_xlpm.fr,VALUE(MID($B21,1,1)),_xlpm.fc,VALUE(MID($B21,2,1)),_xlpm.tr,VALUE(MID($B21,3,1)),_xlpm.tc,VALUE(MID($B21,4,1)),_xlpm.pc,INDEX($B$10:$I$17,_xlpm.fr,_xlpm.fc),_xlpm.cp,INDEX($B$10:$I$17,_xlpm.tr,_xlpm.tc),_xlpm.ch,MID($B21,5,1)="1",_xlpm.mt,MID($B21,6,1)="1",_xlpm.st,MID($B21,7,1)="1",_xlpm.nm,xPN(_xlpm.pc),_xlpm.esc,xHANG($B$10:$I$17,_xlpm.fr,_xlpm.fc)&gt;0,_xlpm.ck,IF(_xlpm.ch," with check",""),IF(_xlpm.mt,"Checkmate. "&amp;_xlpm.nm&amp;" to "&amp;$D21&amp;" and there is no legal reply.",IF(_xlpm.st,"Stalemate. Throws the position away, pick another move.",IF(_xlpm.cp&lt;&gt;"",_xlpm.nm&amp;" takes the "&amp;xPN(_xlpm.cp)&amp;" on "&amp;$D21&amp;_xlpm.ck&amp;".",IF(_xlpm.esc,_xlpm.nm&amp;" escapes "&amp;$C21&amp;", where it can be taken, and goes to "&amp;$D21&amp;_xlpm.ck&amp;".",IF(_xlpm.ch,_xlpm.nm&amp;" "&amp;$C21&amp;" to "&amp;$D21&amp;" gives check.",_xlpm.nm&amp;" "&amp;$C21&amp;" to "&amp;$D21&amp;".")))))))</f>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="38">
-        <v>2</v>
-      </c>
-      <c r="B22" s="38">
-        <f ca="1">IF(LEN($L$7)&gt;=$A22*14,MID($L$7,($A22-1)*14+1,14),"")</f>
-      </c>
-      <c r="C22" s="38">
-        <f ca="1">IF($B22="","",xSQ(VALUE(MID($B22,1,1)),VALUE(MID($B22,2,1))))</f>
-      </c>
-      <c r="D22" s="38">
-        <f ca="1">IF($B22="","",xSQ(VALUE(MID($B22,3,1)),VALUE(MID($B22,4,1))))</f>
-      </c>
-      <c r="E22" s="38">
-        <f ca="1">IF($B22="","",xPN(INDEX($B$10:$I$17,VALUE(MID($B22,1,1)),VALUE(MID($B22,2,1)))))</f>
-      </c>
-      <c r="F22" s="38">
-        <f ca="1">IF($B22="","",xGLY(INDEX($B$10:$I$17,VALUE(MID($B22,1,1)),VALUE(MID($B22,2,1)))))</f>
-      </c>
-      <c r="G22" s="44">
-        <f ca="1">IF($B22="","",(VALUE(MID($B22,8,7))-500000)/100)</f>
-      </c>
-      <c r="H22" s="38">
-        <f ca="1">IF($B22="","",IF(MID($B22,6,1)="1","Checkmate",IF(MID($B22,7,1)="1","Stalemate",IF(MID($B22,5,1)="1","Check",IF(INDEX($B$10:$I$17,VALUE(MID($B22,3,1)),VALUE(MID($B22,4,1)))&lt;&gt;"","Capture","Quiet")))))</f>
-      </c>
-      <c r="I22" s="38">
-        <f ca="1">IF($B22="","",_xlfn.LET(_xlpm.fr,VALUE(MID($B22,1,1)),_xlpm.fc,VALUE(MID($B22,2,1)),_xlpm.tr,VALUE(MID($B22,3,1)),_xlpm.tc,VALUE(MID($B22,4,1)),_xlpm.pc,INDEX($B$10:$I$17,_xlpm.fr,_xlpm.fc),_xlpm.cp,INDEX($B$10:$I$17,_xlpm.tr,_xlpm.tc),_xlpm.ch,MID($B22,5,1)="1",_xlpm.mt,MID($B22,6,1)="1",_xlpm.st,MID($B22,7,1)="1",_xlpm.nm,xPN(_xlpm.pc),_xlpm.esc,xHANG($B$10:$I$17,_xlpm.fr,_xlpm.fc)&gt;0,_xlpm.ck,IF(_xlpm.ch," with check",""),IF(_xlpm.mt,"Checkmate. "&amp;_xlpm.nm&amp;" to "&amp;$D22&amp;" and there is no legal reply.",IF(_xlpm.st,"Stalemate. Throws the position away, pick another move.",IF(_xlpm.cp&lt;&gt;"",_xlpm.nm&amp;" takes the "&amp;xPN(_xlpm.cp)&amp;" on "&amp;$D22&amp;_xlpm.ck&amp;".",IF(_xlpm.esc,_xlpm.nm&amp;" escapes "&amp;$C22&amp;", where it can be taken, and goes to "&amp;$D22&amp;_xlpm.ck&amp;".",IF(_xlpm.ch,_xlpm.nm&amp;" "&amp;$C22&amp;" to "&amp;$D22&amp;" gives check.",_xlpm.nm&amp;" "&amp;$C22&amp;" to "&amp;$D22&amp;".")))))))</f>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="38">
-        <v>3</v>
-      </c>
-      <c r="B23" s="38">
-        <f ca="1">IF(LEN($L$7)&gt;=$A23*14,MID($L$7,($A23-1)*14+1,14),"")</f>
-      </c>
-      <c r="C23" s="38">
-        <f ca="1">IF($B23="","",xSQ(VALUE(MID($B23,1,1)),VALUE(MID($B23,2,1))))</f>
-      </c>
-      <c r="D23" s="38">
-        <f ca="1">IF($B23="","",xSQ(VALUE(MID($B23,3,1)),VALUE(MID($B23,4,1))))</f>
-      </c>
-      <c r="E23" s="38">
-        <f ca="1">IF($B23="","",xPN(INDEX($B$10:$I$17,VALUE(MID($B23,1,1)),VALUE(MID($B23,2,1)))))</f>
-      </c>
-      <c r="F23" s="38">
-        <f ca="1">IF($B23="","",xGLY(INDEX($B$10:$I$17,VALUE(MID($B23,1,1)),VALUE(MID($B23,2,1)))))</f>
-      </c>
-      <c r="G23" s="44">
-        <f ca="1">IF($B23="","",(VALUE(MID($B23,8,7))-500000)/100)</f>
-      </c>
-      <c r="H23" s="38">
-        <f ca="1">IF($B23="","",IF(MID($B23,6,1)="1","Checkmate",IF(MID($B23,7,1)="1","Stalemate",IF(MID($B23,5,1)="1","Check",IF(INDEX($B$10:$I$17,VALUE(MID($B23,3,1)),VALUE(MID($B23,4,1)))&lt;&gt;"","Capture","Quiet")))))</f>
-      </c>
-      <c r="I23" s="38">
-        <f ca="1">IF($B23="","",_xlfn.LET(_xlpm.fr,VALUE(MID($B23,1,1)),_xlpm.fc,VALUE(MID($B23,2,1)),_xlpm.tr,VALUE(MID($B23,3,1)),_xlpm.tc,VALUE(MID($B23,4,1)),_xlpm.pc,INDEX($B$10:$I$17,_xlpm.fr,_xlpm.fc),_xlpm.cp,INDEX($B$10:$I$17,_xlpm.tr,_xlpm.tc),_xlpm.ch,MID($B23,5,1)="1",_xlpm.mt,MID($B23,6,1)="1",_xlpm.st,MID($B23,7,1)="1",_xlpm.nm,xPN(_xlpm.pc),_xlpm.esc,xHANG($B$10:$I$17,_xlpm.fr,_xlpm.fc)&gt;0,_xlpm.ck,IF(_xlpm.ch," with check",""),IF(_xlpm.mt,"Checkmate. "&amp;_xlpm.nm&amp;" to "&amp;$D23&amp;" and there is no legal reply.",IF(_xlpm.st,"Stalemate. Throws the position away, pick another move.",IF(_xlpm.cp&lt;&gt;"",_xlpm.nm&amp;" takes the "&amp;xPN(_xlpm.cp)&amp;" on "&amp;$D23&amp;_xlpm.ck&amp;".",IF(_xlpm.esc,_xlpm.nm&amp;" escapes "&amp;$C23&amp;", where it can be taken, and goes to "&amp;$D23&amp;_xlpm.ck&amp;".",IF(_xlpm.ch,_xlpm.nm&amp;" "&amp;$C23&amp;" to "&amp;$D23&amp;" gives check.",_xlpm.nm&amp;" "&amp;$C23&amp;" to "&amp;$D23&amp;".")))))))</f>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="38">
-        <v>4</v>
-      </c>
-      <c r="B24" s="38">
-        <f ca="1">IF(LEN($L$7)&gt;=$A24*14,MID($L$7,($A24-1)*14+1,14),"")</f>
-      </c>
-      <c r="C24" s="38">
-        <f ca="1">IF($B24="","",xSQ(VALUE(MID($B24,1,1)),VALUE(MID($B24,2,1))))</f>
-      </c>
-      <c r="D24" s="38">
-        <f ca="1">IF($B24="","",xSQ(VALUE(MID($B24,3,1)),VALUE(MID($B24,4,1))))</f>
-      </c>
-      <c r="E24" s="38">
-        <f ca="1">IF($B24="","",xPN(INDEX($B$10:$I$17,VALUE(MID($B24,1,1)),VALUE(MID($B24,2,1)))))</f>
-      </c>
-      <c r="F24" s="38">
-        <f ca="1">IF($B24="","",xGLY(INDEX($B$10:$I$17,VALUE(MID($B24,1,1)),VALUE(MID($B24,2,1)))))</f>
-      </c>
-      <c r="G24" s="44">
-        <f ca="1">IF($B24="","",(VALUE(MID($B24,8,7))-500000)/100)</f>
-      </c>
-      <c r="H24" s="38">
-        <f ca="1">IF($B24="","",IF(MID($B24,6,1)="1","Checkmate",IF(MID($B24,7,1)="1","Stalemate",IF(MID($B24,5,1)="1","Check",IF(INDEX($B$10:$I$17,VALUE(MID($B24,3,1)),VALUE(MID($B24,4,1)))&lt;&gt;"","Capture","Quiet")))))</f>
-      </c>
-      <c r="I24" s="38">
-        <f ca="1">IF($B24="","",_xlfn.LET(_xlpm.fr,VALUE(MID($B24,1,1)),_xlpm.fc,VALUE(MID($B24,2,1)),_xlpm.tr,VALUE(MID($B24,3,1)),_xlpm.tc,VALUE(MID($B24,4,1)),_xlpm.pc,INDEX($B$10:$I$17,_xlpm.fr,_xlpm.fc),_xlpm.cp,INDEX($B$10:$I$17,_xlpm.tr,_xlpm.tc),_xlpm.ch,MID($B24,5,1)="1",_xlpm.mt,MID($B24,6,1)="1",_xlpm.st,MID($B24,7,1)="1",_xlpm.nm,xPN(_xlpm.pc),_xlpm.esc,xHANG($B$10:$I$17,_xlpm.fr,_xlpm.fc)&gt;0,_xlpm.ck,IF(_xlpm.ch," with check",""),IF(_xlpm.mt,"Checkmate. "&amp;_xlpm.nm&amp;" to "&amp;$D24&amp;" and there is no legal reply.",IF(_xlpm.st,"Stalemate. Throws the position away, pick another move.",IF(_xlpm.cp&lt;&gt;"",_xlpm.nm&amp;" takes the "&amp;xPN(_xlpm.cp)&amp;" on "&amp;$D24&amp;_xlpm.ck&amp;".",IF(_xlpm.esc,_xlpm.nm&amp;" escapes "&amp;$C24&amp;", where it can be taken, and goes to "&amp;$D24&amp;_xlpm.ck&amp;".",IF(_xlpm.ch,_xlpm.nm&amp;" "&amp;$C24&amp;" to "&amp;$D24&amp;" gives check.",_xlpm.nm&amp;" "&amp;$C24&amp;" to "&amp;$D24&amp;".")))))))</f>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="38">
-        <v>5</v>
-      </c>
-      <c r="B25" s="38">
-        <f ca="1">IF(LEN($L$7)&gt;=$A25*14,MID($L$7,($A25-1)*14+1,14),"")</f>
-      </c>
-      <c r="C25" s="38">
-        <f ca="1">IF($B25="","",xSQ(VALUE(MID($B25,1,1)),VALUE(MID($B25,2,1))))</f>
-      </c>
-      <c r="D25" s="38">
-        <f ca="1">IF($B25="","",xSQ(VALUE(MID($B25,3,1)),VALUE(MID($B25,4,1))))</f>
-      </c>
-      <c r="E25" s="38">
-        <f ca="1">IF($B25="","",xPN(INDEX($B$10:$I$17,VALUE(MID($B25,1,1)),VALUE(MID($B25,2,1)))))</f>
-      </c>
-      <c r="F25" s="38">
-        <f ca="1">IF($B25="","",xGLY(INDEX($B$10:$I$17,VALUE(MID($B25,1,1)),VALUE(MID($B25,2,1)))))</f>
-      </c>
-      <c r="G25" s="44">
-        <f ca="1">IF($B25="","",(VALUE(MID($B25,8,7))-500000)/100)</f>
-      </c>
-      <c r="H25" s="38">
-        <f ca="1">IF($B25="","",IF(MID($B25,6,1)="1","Checkmate",IF(MID($B25,7,1)="1","Stalemate",IF(MID($B25,5,1)="1","Check",IF(INDEX($B$10:$I$17,VALUE(MID($B25,3,1)),VALUE(MID($B25,4,1)))&lt;&gt;"","Capture","Quiet")))))</f>
-      </c>
-      <c r="I25" s="38">
-        <f ca="1">IF($B25="","",_xlfn.LET(_xlpm.fr,VALUE(MID($B25,1,1)),_xlpm.fc,VALUE(MID($B25,2,1)),_xlpm.tr,VALUE(MID($B25,3,1)),_xlpm.tc,VALUE(MID($B25,4,1)),_xlpm.pc,INDEX($B$10:$I$17,_xlpm.fr,_xlpm.fc),_xlpm.cp,INDEX($B$10:$I$17,_xlpm.tr,_xlpm.tc),_xlpm.ch,MID($B25,5,1)="1",_xlpm.mt,MID($B25,6,1)="1",_xlpm.st,MID($B25,7,1)="1",_xlpm.nm,xPN(_xlpm.pc),_xlpm.esc,xHANG($B$10:$I$17,_xlpm.fr,_xlpm.fc)&gt;0,_xlpm.ck,IF(_xlpm.ch," with check",""),IF(_xlpm.mt,"Checkmate. "&amp;_xlpm.nm&amp;" to "&amp;$D25&amp;" and there is no legal reply.",IF(_xlpm.st,"Stalemate. Throws the position away, pick another move.",IF(_xlpm.cp&lt;&gt;"",_xlpm.nm&amp;" takes the "&amp;xPN(_xlpm.cp)&amp;" on "&amp;$D25&amp;_xlpm.ck&amp;".",IF(_xlpm.esc,_xlpm.nm&amp;" escapes "&amp;$C25&amp;", where it can be taken, and goes to "&amp;$D25&amp;_xlpm.ck&amp;".",IF(_xlpm.ch,_xlpm.nm&amp;" "&amp;$C25&amp;" to "&amp;$D25&amp;" gives check.",_xlpm.nm&amp;" "&amp;$C25&amp;" to "&amp;$D25&amp;".")))))))</f>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="38">
-        <v>6</v>
-      </c>
-      <c r="B26" s="38">
-        <f ca="1">IF(LEN($L$7)&gt;=$A26*14,MID($L$7,($A26-1)*14+1,14),"")</f>
-      </c>
-      <c r="C26" s="38">
-        <f ca="1">IF($B26="","",xSQ(VALUE(MID($B26,1,1)),VALUE(MID($B26,2,1))))</f>
-      </c>
-      <c r="D26" s="38">
-        <f ca="1">IF($B26="","",xSQ(VALUE(MID($B26,3,1)),VALUE(MID($B26,4,1))))</f>
-      </c>
-      <c r="E26" s="38">
-        <f ca="1">IF($B26="","",xPN(INDEX($B$10:$I$17,VALUE(MID($B26,1,1)),VALUE(MID($B26,2,1)))))</f>
-      </c>
-      <c r="F26" s="38">
-        <f ca="1">IF($B26="","",xGLY(INDEX($B$10:$I$17,VALUE(MID($B26,1,1)),VALUE(MID($B26,2,1)))))</f>
-      </c>
-      <c r="G26" s="44">
-        <f ca="1">IF($B26="","",(VALUE(MID($B26,8,7))-500000)/100)</f>
-      </c>
-      <c r="H26" s="38">
-        <f ca="1">IF($B26="","",IF(MID($B26,6,1)="1","Checkmate",IF(MID($B26,7,1)="1","Stalemate",IF(MID($B26,5,1)="1","Check",IF(INDEX($B$10:$I$17,VALUE(MID($B26,3,1)),VALUE(MID($B26,4,1)))&lt;&gt;"","Capture","Quiet")))))</f>
-      </c>
-      <c r="I26" s="38">
-        <f ca="1">IF($B26="","",_xlfn.LET(_xlpm.fr,VALUE(MID($B26,1,1)),_xlpm.fc,VALUE(MID($B26,2,1)),_xlpm.tr,VALUE(MID($B26,3,1)),_xlpm.tc,VALUE(MID($B26,4,1)),_xlpm.pc,INDEX($B$10:$I$17,_xlpm.fr,_xlpm.fc),_xlpm.cp,INDEX($B$10:$I$17,_xlpm.tr,_xlpm.tc),_xlpm.ch,MID($B26,5,1)="1",_xlpm.mt,MID($B26,6,1)="1",_xlpm.st,MID($B26,7,1)="1",_xlpm.nm,xPN(_xlpm.pc),_xlpm.esc,xHANG($B$10:$I$17,_xlpm.fr,_xlpm.fc)&gt;0,_xlpm.ck,IF(_xlpm.ch," with check",""),IF(_xlpm.mt,"Checkmate. "&amp;_xlpm.nm&amp;" to "&amp;$D26&amp;" and there is no legal reply.",IF(_xlpm.st,"Stalemate. Throws the position away, pick another move.",IF(_xlpm.cp&lt;&gt;"",_xlpm.nm&amp;" takes the "&amp;xPN(_xlpm.cp)&amp;" on "&amp;$D26&amp;_xlpm.ck&amp;".",IF(_xlpm.esc,_xlpm.nm&amp;" escapes "&amp;$C26&amp;", where it can be taken, and goes to "&amp;$D26&amp;_xlpm.ck&amp;".",IF(_xlpm.ch,_xlpm.nm&amp;" "&amp;$C26&amp;" to "&amp;$D26&amp;" gives check.",_xlpm.nm&amp;" "&amp;$C26&amp;" to "&amp;$D26&amp;".")))))))</f>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>